<commit_message>
Tabela 17 com calibração sobre o posto e teste da datação da RJ
- Script 14: métricas de probabilidade com calibração logística sobre o
  posto, nos dois horizontes, com especificidade, VPN e decisão líquida
- Script 15: RJ antecipada em um ano para as 22 firmas com primeiro
  documento de andamento; reconstrução verificada contra os painéis
- Artigo revisado: Tabela 17, §5.7, §5.9, §5.5 e conclusão atualizados
  (103 alterações controladas); planilha com a Tabela 17 completa
- executar.sh roda os 15 scripts e limita threads do OpenMP

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4LwoZDLWB9PeJtPghPCix
</commit_message>
<xml_diff>
--- a/projeto/tabelas/Tabelas_Artigo_revisado.xlsx
+++ b/projeto/tabelas/Tabelas_Artigo_revisado.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estabilidade_h2" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T14_puros" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T15_perfil" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T17_revisada" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -34,7 +35,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -84,6 +85,9 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -127,7 +131,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -195,6 +199,8 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -704,7 +710,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Fonte: 01 e 02. Validação cruzada agrupada por firma, atribuição de referência. Diferença por fórmula. p ajustado por Bonferroni para as seis comparações contra benchmarks e referência não linear; a comparação com mínimos quadrados parciais responde a H4 e não é ajustada.</t>
         </is>
@@ -1929,6 +1935,722 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="12" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>Tabela 17 (revisada) – Métricas de probabilidade e desempenho operacional, calibração sobre o posto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Horizonte</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>AUC precisão-revocação</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>Brier</t>
+        </is>
+      </c>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Inclinação</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>Intercepto</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>Sensibilidade</t>
+        </is>
+      </c>
+      <c r="H2" s="23" t="inlineStr">
+        <is>
+          <t>Especificidade</t>
+        </is>
+      </c>
+      <c r="I2" s="23" t="inlineStr">
+        <is>
+          <t>VPP</t>
+        </is>
+      </c>
+      <c r="J2" s="23" t="inlineStr">
+        <is>
+          <t>VPN</t>
+        </is>
+      </c>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>Firma-anos sinalizados</t>
+        </is>
+      </c>
+      <c r="L2" s="23" t="inlineStr">
+        <is>
+          <t>Decisão líquida 5:1</t>
+        </is>
+      </c>
+      <c r="M2" s="23" t="inlineStr">
+        <is>
+          <t>Decisão líquida 10:1</t>
+        </is>
+      </c>
+      <c r="N2" s="23" t="inlineStr">
+        <is>
+          <t>Decisão líquida 20:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Árvores impulsionadas</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="n">
+        <v>0.2295344679757571</v>
+      </c>
+      <c r="D3" s="24" t="n">
+        <v>0.02506581222288731</v>
+      </c>
+      <c r="E3" s="24" t="n">
+        <v>1.086640234786473</v>
+      </c>
+      <c r="F3" s="24" t="n">
+        <v>-0.02831372516967114</v>
+      </c>
+      <c r="G3" s="24" t="n">
+        <v>0.785234899328859</v>
+      </c>
+      <c r="H3" s="24" t="n">
+        <v>0.8462323871758219</v>
+      </c>
+      <c r="I3" s="24" t="n">
+        <v>0.1344827586206896</v>
+      </c>
+      <c r="J3" s="24" t="n">
+        <v>0.9923371647509579</v>
+      </c>
+      <c r="K3" s="24" t="n">
+        <v>0.1724137931034483</v>
+      </c>
+      <c r="L3" s="24" t="n">
+        <v>0.006024573919936584</v>
+      </c>
+      <c r="M3" s="24" t="n">
+        <v>0.01080063416567578</v>
+      </c>
+      <c r="N3" s="24" t="n">
+        <v>0.01603250099088387</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cobertura de juros</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="n">
+        <v>0.1844374990629637</v>
+      </c>
+      <c r="D4" s="24" t="n">
+        <v>0.02561585837572898</v>
+      </c>
+      <c r="E4" s="24" t="n">
+        <v>0.9879690002439582</v>
+      </c>
+      <c r="F4" s="24" t="n">
+        <v>-0.004322604940026632</v>
+      </c>
+      <c r="G4" s="24" t="n">
+        <v>0.785234899328859</v>
+      </c>
+      <c r="H4" s="24" t="n">
+        <v>0.8311210945476822</v>
+      </c>
+      <c r="I4" s="24" t="n">
+        <v>0.1239406779661017</v>
+      </c>
+      <c r="J4" s="24" t="n">
+        <v>0.9921989273525109</v>
+      </c>
+      <c r="K4" s="24" t="n">
+        <v>0.1870788743559255</v>
+      </c>
+      <c r="L4" s="24" t="n">
+        <v>0.002695204122076893</v>
+      </c>
+      <c r="M4" s="24" t="n">
+        <v>0.009274673008323424</v>
+      </c>
+      <c r="N4" s="24" t="n">
+        <v>0.01489298454221165</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Retorno sobre ativos</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>0.1753661270949595</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>0.02597582725174593</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>0.9931475518719396</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>-0.004774228210969339</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>0.7919463087248322</v>
+      </c>
+      <c r="H5" s="24" t="n">
+        <v>0.8427608740044925</v>
+      </c>
+      <c r="I5" s="24" t="n">
+        <v>0.1328828828828829</v>
+      </c>
+      <c r="J5" s="24" t="n">
+        <v>0.9925444925444925</v>
+      </c>
+      <c r="K5" s="24" t="n">
+        <v>0.1759809750297265</v>
+      </c>
+      <c r="L5" s="24" t="n">
+        <v>0.002695204122076893</v>
+      </c>
+      <c r="M5" s="24" t="n">
+        <v>0.008997225525168448</v>
+      </c>
+      <c r="N5" s="24" t="n">
+        <v>0.01546769718588981</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mínimos quadrados parciais</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>0.1719750799692672</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>0.02603112214350956</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>1.07206022415256</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>0.007250948427309378</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>0.7919463087248322</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>0.8100878088625689</v>
+      </c>
+      <c r="I6" s="24" t="n">
+        <v>0.1125954198473282</v>
+      </c>
+      <c r="J6" s="24" t="n">
+        <v>0.9922461230615308</v>
+      </c>
+      <c r="K6" s="24" t="n">
+        <v>0.2076892588188664</v>
+      </c>
+      <c r="L6" s="24" t="n">
+        <v>0.002338485929449069</v>
+      </c>
+      <c r="M6" s="24" t="n">
+        <v>0.008085612366230677</v>
+      </c>
+      <c r="N6" s="24" t="n">
+        <v>0.01439754260800634</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Componentes principais (F)</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n">
+        <v>0.1112965384710407</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>0.02752650275823896</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>0.9913595502153402</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>-0.005980251387520434</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>0.7986577181208053</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <v>0.5699407800694303</v>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>0.05348314606741573</v>
+      </c>
+      <c r="J7" s="24" t="n">
+        <v>0.989365473236441</v>
+      </c>
+      <c r="K7" s="24" t="n">
+        <v>0.4409433214427269</v>
+      </c>
+      <c r="L7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="24" t="n">
+        <v>0.003032104637336504</v>
+      </c>
+      <c r="N7" s="24" t="n">
+        <v>0.008531510107015458</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Brito e Assaf Neto</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>0.09476579481990252</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>0.02777774711172786</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>1.075469920058045</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>0.01462486734399807</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>0.8187919463087249</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>0.4617112517868083</v>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>0.04423495286439449</v>
+      </c>
+      <c r="J8" s="24" t="n">
+        <v>0.9881993006993007</v>
+      </c>
+      <c r="K8" s="24" t="n">
+        <v>0.5465715418152992</v>
+      </c>
+      <c r="L8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="24" t="n">
+        <v>0.001149425287356322</v>
+      </c>
+      <c r="N8" s="24" t="n">
+        <v>0.009373761395164486</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1 ano</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Referência sem informação</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>0.02952833927863655</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>0.02865641645808228</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Árvores impulsionadas</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>0.08521677951450135</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>0.02766025850960952</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>1.158922573673336</v>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>-0.06657935493350987</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>0.4992802303262956</v>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>0.0479014598540146</v>
+      </c>
+      <c r="J10" s="24" t="n">
+        <v>0.9900095147478591</v>
+      </c>
+      <c r="K10" s="24" t="n">
+        <v>0.5104797391709361</v>
+      </c>
+      <c r="L10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="24" t="n">
+        <v>0.0003493246390312063</v>
+      </c>
+      <c r="N10" s="24" t="n">
+        <v>0.00716115510013973</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cobertura de juros</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>0.05062672744829048</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>0.02815802062181195</v>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>0.9483481095724542</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <v>-0.004682623198508686</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>0.8015873015873016</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <v>0.4517754318618042</v>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>0.04233025984911987</v>
+      </c>
+      <c r="J11" s="24" t="n">
+        <v>0.9868972746331237</v>
+      </c>
+      <c r="K11" s="24" t="n">
+        <v>0.5556590591523055</v>
+      </c>
+      <c r="L11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="24" t="n">
+        <v>0.003446669771774569</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Retorno sobre ativos</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>0.0657719994412717</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>0.02788264124527806</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>0.9751588747917186</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>-0.002241119276739794</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>0.8015873015873016</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>0.5890115163147792</v>
+      </c>
+      <c r="I12" s="24" t="n">
+        <v>0.05567805953693495</v>
+      </c>
+      <c r="J12" s="24" t="n">
+        <v>0.9899193548387096</v>
+      </c>
+      <c r="K12" s="24" t="n">
+        <v>0.4224499301350722</v>
+      </c>
+      <c r="L12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="24" t="n">
+        <v>-0.0006054960409874245</v>
+      </c>
+      <c r="N12" s="24" t="n">
+        <v>0.004413134606427572</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mínimos quadrados parciais</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>0.0644946967358081</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>0.02788026651722164</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>1.075412988199589</v>
+      </c>
+      <c r="F13" s="24" t="n">
+        <v>-0.008215222846687494</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>0.7936507936507936</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <v>0.5328694817658349</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>0.04885197850512946</v>
+      </c>
+      <c r="J13" s="24" t="n">
+        <v>0.9884290164663997</v>
+      </c>
+      <c r="K13" s="24" t="n">
+        <v>0.4767116907312529</v>
+      </c>
+      <c r="L13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="24" t="n">
+        <v>-0.000232883092687471</v>
+      </c>
+      <c r="N13" s="24" t="n">
+        <v>0.006590591523055425</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Componentes principais (F)</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>0.05391257689226329</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>0.02829360358512675</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <v>0.9153978808503124</v>
+      </c>
+      <c r="F14" s="24" t="n">
+        <v>-0.001851267795798534</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>0.7936507936507936</v>
+      </c>
+      <c r="H14" s="24" t="n">
+        <v>0.2881477927063339</v>
+      </c>
+      <c r="I14" s="24" t="n">
+        <v>0.032605151613955</v>
+      </c>
+      <c r="J14" s="24" t="n">
+        <v>0.9788101059494703</v>
+      </c>
+      <c r="K14" s="24" t="n">
+        <v>0.7142524452724732</v>
+      </c>
+      <c r="L14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="24" t="n">
+        <v>0.003435025617140196</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Brito e Assaf Neto</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>0.06037014219553517</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>0.02812598530144687</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>1.260703044771871</v>
+      </c>
+      <c r="F15" s="24" t="n">
+        <v>-0.008544417368427756</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>0.8492063492063492</v>
+      </c>
+      <c r="H15" s="24" t="n">
+        <v>0.2922264875239923</v>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>0.03500163559044815</v>
+      </c>
+      <c r="J15" s="24" t="n">
+        <v>0.98464025869038</v>
+      </c>
+      <c r="K15" s="24" t="n">
+        <v>0.7119236143455985</v>
+      </c>
+      <c r="L15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="24" t="n">
+        <v>0.004843968327899395</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2 anos</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Referência sem informação</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>0.02934326967862133</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>0.02848224220318903</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fonte: script 14. Calibração logística sobre o posto do escore na distribuição do treino; limiar que atinge sensibilidade de 80% nas firmas de treino, aplicado às de teste. Decisão líquida por firma-ano; a de não sinalizar ninguém é zero.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -2191,7 +2913,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Fonte: 01 e 02. Validação cruzada agrupada por firma, atribuição de referência. Diferença por fórmula. p ajustado por Bonferroni para as seis comparações contra benchmarks e referência não linear; a comparação com mínimos quadrados parciais responde a H4 e não é ajustada.</t>
         </is>

</xml_diff>

<commit_message>
Fecha pendências da revisão: saídas pelo cadastro, literatura, figuras e verificação automática
- Saídas: composição pelo cadastro da CVM e sensibilidade como risco
  competitivo (Tabela 19, linha nova)
- Árvores alinhadas à versão fixada em todas as tabelas, texto e figuras;
  Ponzi exige exercícios consecutivos; coluna MEB na Tabela 13
- Estabilidade entre atribuições reportada (prometida e ausente)
- Afirmações sobre 20 obras conferidas na fonte; 13 correções
- Planilha preenchida pelo código final; nota de decisões revisada;
  registro bibliográfico com 45 entradas
- Verificador automático: 584 células das tabelas conferidas contra o
  código, sem divergência (controle no original acusa as 50 corrigidas)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4LwoZDLWB9PeJtPghPCix
</commit_message>
<xml_diff>
--- a/projeto/tabelas/Tabelas_Artigo_revisado.xlsx
+++ b/projeto/tabelas/Tabelas_Artigo_revisado.xlsx
@@ -20,7 +20,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estabilidade_h2" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T14_puros" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T15_perfil" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T17_revisada" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -131,7 +130,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -187,6 +186,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
@@ -199,8 +199,6 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +510,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>0.764267398338662</v>
+        <v>0.7642673983386623</v>
       </c>
       <c r="C4" s="17" t="n"/>
       <c r="D4" s="17" t="n"/>
@@ -527,17 +525,17 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.900185430608796</v>
+        <v>0.8969839087895205</v>
       </c>
       <c r="C5" s="17">
         <f>B5-$B$4</f>
         <v/>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.09024207789425299</v>
+        <v>0.0857751707434312</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.183902588858983</v>
+        <v>0.1813942265915912</v>
       </c>
       <c r="F5" s="16" t="n">
         <v>0.0005</v>
@@ -554,7 +552,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.893687136214063</v>
+        <v>0.8936871362140634</v>
       </c>
       <c r="C6" s="17">
         <f>B6-$B$4</f>
@@ -564,7 +562,7 @@
         <v>0.0800957193667922</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.181328875610143</v>
+        <v>0.1813288756101432</v>
       </c>
       <c r="F6" s="16" t="n">
         <v>0.0005</v>
@@ -581,7 +579,7 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.875253031235395</v>
+        <v>0.8752530312353954</v>
       </c>
       <c r="C7" s="17">
         <f>B7-$B$4</f>
@@ -591,7 +589,7 @@
         <v>0.0644198867522225</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.160335239951334</v>
+        <v>0.1603352399513336</v>
       </c>
       <c r="F7" s="16" t="n">
         <v>0.0005</v>
@@ -608,7 +606,7 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.873875664185579</v>
+        <v>0.8738756641855786</v>
       </c>
       <c r="C8" s="17">
         <f>B8-$B$4</f>
@@ -618,7 +616,7 @@
         <v>0.0607085903949829</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.157800455395518</v>
+        <v>0.1578004553955183</v>
       </c>
       <c r="F8" s="16" t="n">
         <v>0.0005</v>
@@ -635,7 +633,7 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>0.734498453374412</v>
+        <v>0.7344984533744122</v>
       </c>
       <c r="C9" s="17">
         <f>B9-$B$4</f>
@@ -662,7 +660,7 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>0.603972025058487</v>
+        <v>0.6039720250584867</v>
       </c>
       <c r="C10" s="17">
         <f>B10-$B$4</f>
@@ -672,7 +670,7 @@
         <v>-0.193073361694687</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>-0.125432678801339</v>
+        <v>-0.1254326788013387</v>
       </c>
       <c r="F10" s="16" t="n">
         <v>0.0005</v>
@@ -689,17 +687,17 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>0.531137403669964</v>
+        <v>0.5311374036699636</v>
       </c>
       <c r="C11" s="17">
         <f>B11-$B$4</f>
         <v/>
       </c>
       <c r="D11" s="17" t="n">
-        <v>-0.281592099154262</v>
+        <v>-0.2815920991542617</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>-0.181285615837411</v>
+        <v>-0.1812856158374114</v>
       </c>
       <c r="F11" s="16" t="n">
         <v>0.0005</v>
@@ -710,18 +708,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Fonte: 01 e 02. Validação cruzada agrupada por firma, atribuição de referência. Diferença por fórmula. p ajustado por Bonferroni para as seis comparações contra benchmarks e referência não linear; a comparação com mínimos quadrados parciais responde a H4 e não é ajustada.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Fonte: 01 e 02. Validação cruzada agrupada por firma, atribuição de referência. Diferença e p ajustado por fórmula.</t>
-        </is>
-      </c>
+      <c r="A13" s="18" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -789,16 +783,16 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>0.764267398338662</v>
+        <v>0.7642673983386623</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>0.875253031235395</v>
+        <v>0.8752530312353954</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>0.900185430608796</v>
+        <v>0.8969839087895205</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>0.734498453374412</v>
+        <v>0.7344984533744122</v>
       </c>
       <c r="F4" s="17">
         <f>C4-B4</f>
@@ -812,16 +806,16 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.764651142392343</v>
+        <v>0.7646511423923427</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>0.874724012647108</v>
+        <v>0.8747240126471076</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>0.891410711667053</v>
+        <v>0.8904170886709162</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>0.739110234590963</v>
+        <v>0.7391102345909631</v>
       </c>
       <c r="F5" s="17">
         <f>C5-B5</f>
@@ -835,16 +829,16 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.761212521568472</v>
+        <v>0.7612125215684716</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.874192253029865</v>
+        <v>0.8741922530298649</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.90335611585233</v>
+        <v>0.905770962361561</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.73342808156754</v>
+        <v>0.7334280815675397</v>
       </c>
       <c r="F6" s="17">
         <f>C6-B6</f>
@@ -858,16 +852,16 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.762180104789537</v>
+        <v>0.7621801047895369</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>0.877347177356908</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>0.895519514070387</v>
+        <v>0.8955866692797809</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>0.733607618964083</v>
+        <v>0.7336076189640829</v>
       </c>
       <c r="F7" s="17">
         <f>C7-B7</f>
@@ -881,16 +875,16 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.765218535385999</v>
+        <v>0.7652185353859986</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.868708824605669</v>
+        <v>0.8687088246056687</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>0.891981530946902</v>
+        <v>0.8922378171541815</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>0.705465474684542</v>
+        <v>0.7054654746845418</v>
       </c>
       <c r="F8" s="17">
         <f>C8-B8</f>
@@ -904,16 +898,16 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>0.762594000161721</v>
+        <v>0.7625940001617207</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.875088569498104</v>
+        <v>0.8750885694981039</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>0.897446457425653</v>
+        <v>0.9002519005609516</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>0.7277130361966579</v>
+        <v>0.7277130361966578</v>
       </c>
       <c r="F9" s="17">
         <f>C9-B9</f>
@@ -927,16 +921,16 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>0.760266866579045</v>
+        <v>0.7602668665790451</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.870086191655486</v>
+        <v>0.8700861916554855</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.8983749809841119</v>
+        <v>0.8994330181606873</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.725224181905646</v>
+        <v>0.7252241819056455</v>
       </c>
       <c r="F10" s="17">
         <f>C10-B10</f>
@@ -950,16 +944,16 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>0.7638192401045431</v>
+        <v>0.7638192401045428</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>0.875402417313435</v>
+        <v>0.8754024173134353</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>0.898148846095336</v>
+        <v>0.8989204457461286</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>0.731634078116584</v>
+        <v>0.7316340781165842</v>
       </c>
       <c r="F11" s="17">
         <f>C11-B11</f>
@@ -973,16 +967,16 @@
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>0.764874536252164</v>
+        <v>0.7648745362521637</v>
       </c>
       <c r="C12" s="16" t="n">
         <v>0.876013666770369</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.895207722026772</v>
+        <v>0.8942250631464546</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.705920485491049</v>
+        <v>0.7059204854910485</v>
       </c>
       <c r="F12" s="17">
         <f>C12-B12</f>
@@ -996,16 +990,16 @@
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>0.7629928198746529</v>
+        <v>0.7629928198746527</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>0.871410108640683</v>
+        <v>0.8714101086406826</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>0.899316524430106</v>
+        <v>0.8988053225300245</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>0.717530113629355</v>
+        <v>0.7175301136293554</v>
       </c>
       <c r="F13" s="17">
         <f>C13-B13</f>
@@ -1166,13 +1160,13 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>0.6266128172318191</v>
+        <v>0.6266128172318192</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>0.724754745148219</v>
+        <v>0.7247547451482192</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>0.751919385796545</v>
+        <v>0.7525839350455473</v>
       </c>
       <c r="E4" s="16" t="n">
         <v>0.667237912439448</v>
@@ -1189,16 +1183,16 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.626995551899583</v>
+        <v>0.6269955518995826</v>
       </c>
       <c r="C5" s="16" t="n">
         <v>0.720032446759894</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>0.769741301831033</v>
+        <v>0.7710380297352466</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>0.667915790756482</v>
+        <v>0.6679157907564818</v>
       </c>
       <c r="F5" s="17">
         <f>C5-B5</f>
@@ -1212,16 +1206,16 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.625723577978856</v>
+        <v>0.6257235779788562</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.73743830545654</v>
+        <v>0.7374383054565397</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.765351278067209</v>
+        <v>0.7616648386801937</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.667106525911708</v>
+        <v>0.6671065259117083</v>
       </c>
       <c r="F6" s="17">
         <f>C6-B6</f>
@@ -1235,13 +1229,13 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.626254836547543</v>
+        <v>0.6262548365475429</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>0.725828687201048</v>
+        <v>0.7258286872010481</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>0.765650230021631</v>
+        <v>0.7624036498796576</v>
       </c>
       <c r="E7" s="16" t="n">
         <v>0.677398470584651</v>
@@ -1258,16 +1252,16 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.6276353471650979</v>
+        <v>0.6276353471650976</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.723438975718246</v>
+        <v>0.7234389757182463</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>0.751772766048198</v>
+        <v>0.7543909758401122</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>0.665815510465223</v>
+        <v>0.6658155104652226</v>
       </c>
       <c r="F8" s="17">
         <f>C8-B8</f>
@@ -1281,16 +1275,16 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>0.6266623251987939</v>
+        <v>0.6266623251987935</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.723795052249947</v>
+        <v>0.7237950522499467</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>0.745784206196874</v>
+        <v>0.747254211985498</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>0.669239176796758</v>
+        <v>0.6692391767967584</v>
       </c>
       <c r="F9" s="17">
         <f>C9-B9</f>
@@ -1304,16 +1298,16 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>0.626835603083204</v>
+        <v>0.6268356030832039</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.729101925479085</v>
+        <v>0.7291019254790848</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.768146574048685</v>
+        <v>0.7652351247600768</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.670943393352223</v>
+        <v>0.6709433933522225</v>
       </c>
       <c r="F10" s="17">
         <f>C10-B10</f>
@@ -1327,16 +1321,16 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>0.626650900283338</v>
+        <v>0.6266509002833379</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>0.7338584986137771</v>
+        <v>0.7338584986137769</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>0.737755346860433</v>
+        <v>0.7338708756055206</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>0.663745696615178</v>
+        <v>0.6637456966151783</v>
       </c>
       <c r="F11" s="17">
         <f>C11-B11</f>
@@ -1350,16 +1344,16 @@
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>0.628852100661122</v>
+        <v>0.6288521006611217</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.722806797063035</v>
+        <v>0.7228067970630351</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.758155485482741</v>
+        <v>0.7528219541175395</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.653823157541968</v>
+        <v>0.6538231575419675</v>
       </c>
       <c r="F12" s="17">
         <f>C12-B12</f>
@@ -1373,16 +1367,16 @@
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>0.625348459921397</v>
+        <v>0.6253484599213965</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>0.723608445297505</v>
+        <v>0.7236084452975048</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>0.757784175730433</v>
+        <v>0.7529438198823996</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>0.654594339335222</v>
+        <v>0.6545943393352223</v>
       </c>
       <c r="F13" s="17">
         <f>C13-B13</f>
@@ -1557,29 +1551,29 @@
           <t>Prejuízo operacional, um ano</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n">
+      <c r="B4" s="20" t="n">
         <v>66</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>0.648909969616525</v>
+        <v>0.6489099696165247</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>0.324077511896585</v>
+        <v>0.3240775118965847</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>0.244100108700858</v>
+        <v>0.2441001087008582</v>
       </c>
       <c r="F4" s="17" t="n">
-        <v>0.411347735813248</v>
+        <v>0.4113477358132478</v>
       </c>
       <c r="G4" s="17" t="n">
-        <v>0.290647953911176</v>
+        <v>0.2906479539111763</v>
       </c>
       <c r="H4" s="17" t="n">
-        <v>0.21692673915229</v>
+        <v>0.2169267391522895</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>0.371379769878476</v>
+        <v>0.3713797698784761</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -1588,29 +1582,29 @@
           <t>Patrimônio negativo, um ano</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="20" t="n">
         <v>51</v>
       </c>
       <c r="C5" s="16" t="n">
         <v>0.816061854596852</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>-0.0295679227378106</v>
+        <v>-0.02956792273781061</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>-0.0931150860370642</v>
+        <v>-0.09311508603706418</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.0378691176104551</v>
+        <v>0.03786911761045506</v>
       </c>
       <c r="G5" s="17" t="n">
         <v>-0.0658906813695459</v>
       </c>
       <c r="H5" s="17" t="n">
-        <v>-0.128871306387324</v>
+        <v>-0.1288713063873238</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-0.00336011975959002</v>
+        <v>-0.003360119759590024</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
@@ -1619,29 +1613,29 @@
           <t>Recuperação judicial, um ano</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="20" t="n">
         <v>11</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.8277609668257</v>
+        <v>0.8277609668257003</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.0115748046113576</v>
+        <v>0.01157480461135763</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>-0.0966075553574374</v>
+        <v>-0.09660755535743742</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.116685770171869</v>
+        <v>0.1166857701718687</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>0.0627657007072976</v>
+        <v>0.06276570070729759</v>
       </c>
       <c r="H6" s="17" t="n">
-        <v>-0.000664281309838832</v>
+        <v>-0.0006642813098388315</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>0.136326109061503</v>
+        <v>0.1363261090615032</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
@@ -1650,29 +1644,29 @@
           <t>Prejuízo operacional, dois anos</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="20" t="n">
         <v>52</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>0.377496124317142</v>
+        <v>0.3774961243171416</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>0.144636793149269</v>
+        <v>0.1446367931492692</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>0.0572070649833604</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0.23266212297695</v>
+        <v>0.2326621229769502</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>0.275247305477632</v>
+        <v>0.2752473054776318</v>
       </c>
       <c r="H7" s="17" t="n">
-        <v>0.195950480463531</v>
+        <v>0.1959504804635307</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>0.353055807344646</v>
+        <v>0.3530558073446463</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
@@ -1681,26 +1675,26 @@
           <t>Patrimônio negativo, dois anos</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>46</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.795590628390219</v>
+        <v>0.7955906283902194</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>-0.00482193524159225</v>
+        <v>-0.004821935241592246</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>-0.0689285262538219</v>
+        <v>-0.06892852625382186</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>0.0631841407302173</v>
+        <v>0.06318414073021726</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>-0.0824918634732538</v>
+        <v>-0.08249186347325377</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>-0.139293051181214</v>
+        <v>-0.1392930511812144</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>-0.0231236879844152</v>
@@ -1712,29 +1706,29 @@
           <t>Recuperação judicial, dois anos</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="B9" s="20" t="n">
         <v>9</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.800890381744508</v>
+        <v>0.8008903817445084</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>-0.0875986351034336</v>
+        <v>-0.08759863510343358</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>-0.240416027723596</v>
+        <v>-0.2404160277235961</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>0.069014733739918</v>
+        <v>0.06901473373991801</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>0.0533162721262529</v>
+        <v>0.05331627212625289</v>
       </c>
       <c r="H9" s="17" t="n">
-        <v>-0.0261072601981677</v>
+        <v>-0.02610726019816766</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>0.147880759690188</v>
+        <v>0.1478807596901882</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
@@ -1799,13 +1793,13 @@
           <t>Alavancagem</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.213065036228923</v>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="21" t="n">
         <v>0.425126544113893</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.326386397196832</v>
       </c>
     </row>
@@ -1815,13 +1809,13 @@
           <t>Liquidez corrente</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
-        <v>1.99804941015869</v>
-      </c>
-      <c r="C5" s="20" t="n">
+      <c r="B5" s="21" t="n">
+        <v>1.998049410158685</v>
+      </c>
+      <c r="C5" s="21" t="n">
         <v>0.943732022580715</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="21" t="n">
         <v>1.43043910867033</v>
       </c>
     </row>
@@ -1831,13 +1825,13 @@
           <t>Capital de giro sobre ativo</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
-        <v>0.176364759295332</v>
-      </c>
-      <c r="C6" s="20" t="n">
+      <c r="B6" s="21" t="n">
+        <v>0.1763647592953315</v>
+      </c>
+      <c r="C6" s="21" t="n">
         <v>-0.024871125548301</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.084351266928543</v>
       </c>
     </row>
@@ -1847,13 +1841,13 @@
           <t>Cobertura de juros</t>
         </is>
       </c>
-      <c r="B7" s="20" t="n">
-        <v>1.41109589230522</v>
-      </c>
-      <c r="C7" s="20" t="n">
+      <c r="B7" s="21" t="n">
+        <v>1.411095892305215</v>
+      </c>
+      <c r="C7" s="21" t="n">
         <v>0.37655960009212</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="21" t="n">
         <v>1.50992137747865</v>
       </c>
     </row>
@@ -1863,13 +1857,13 @@
           <t>Retorno sobre ativos</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="21" t="n">
         <v>0.0163713580410209</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="21" t="n">
         <v>-0.0336808481906868</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="21" t="n">
         <v>0.0396492206621962</v>
       </c>
     </row>
@@ -1879,13 +1873,13 @@
           <t>Margem EBITDA</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n">
-        <v>0.132044750505732</v>
-      </c>
-      <c r="C9" s="20" t="n">
+      <c r="B9" s="21" t="n">
+        <v>0.1320447505057315</v>
+      </c>
+      <c r="C9" s="21" t="n">
         <v>0.117722059244612</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="21" t="n">
         <v>0.211605259184521</v>
       </c>
     </row>
@@ -1895,13 +1889,13 @@
           <t>Logaritmo do ativo real</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <v>21.5013478037086</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="21" t="n">
         <v>21.4529774714187</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="21" t="n">
         <v>22.1714420501993</v>
       </c>
     </row>
@@ -1911,20 +1905,20 @@
           <t>Observações</t>
         </is>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="21" t="n">
         <v>52</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="21" t="n">
         <v>65</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="21" t="n">
         <v>4193</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Fonte: 13. Horizonte de dois anos, sobre a amostra de risco.</t>
+          <t>Fonte: 13. Horizonte de dois anos, sobre a amostra de risco. A primeira coluna reúne as entradas apenas pelo critério de EBITDA; a segunda, todas as entradas por patrimônio líquido negativo, inclusive as que satisfazem outro critério.</t>
         </is>
       </c>
     </row>
@@ -1932,722 +1926,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" style="12" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="23" t="inlineStr">
-        <is>
-          <t>Tabela 17 (revisada) – Métricas de probabilidade e desempenho operacional, calibração sobre o posto</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>Horizonte</t>
-        </is>
-      </c>
-      <c r="B2" s="23" t="inlineStr">
-        <is>
-          <t>Modelo</t>
-        </is>
-      </c>
-      <c r="C2" s="23" t="inlineStr">
-        <is>
-          <t>AUC precisão-revocação</t>
-        </is>
-      </c>
-      <c r="D2" s="23" t="inlineStr">
-        <is>
-          <t>Brier</t>
-        </is>
-      </c>
-      <c r="E2" s="23" t="inlineStr">
-        <is>
-          <t>Inclinação</t>
-        </is>
-      </c>
-      <c r="F2" s="23" t="inlineStr">
-        <is>
-          <t>Intercepto</t>
-        </is>
-      </c>
-      <c r="G2" s="23" t="inlineStr">
-        <is>
-          <t>Sensibilidade</t>
-        </is>
-      </c>
-      <c r="H2" s="23" t="inlineStr">
-        <is>
-          <t>Especificidade</t>
-        </is>
-      </c>
-      <c r="I2" s="23" t="inlineStr">
-        <is>
-          <t>VPP</t>
-        </is>
-      </c>
-      <c r="J2" s="23" t="inlineStr">
-        <is>
-          <t>VPN</t>
-        </is>
-      </c>
-      <c r="K2" s="23" t="inlineStr">
-        <is>
-          <t>Firma-anos sinalizados</t>
-        </is>
-      </c>
-      <c r="L2" s="23" t="inlineStr">
-        <is>
-          <t>Decisão líquida 5:1</t>
-        </is>
-      </c>
-      <c r="M2" s="23" t="inlineStr">
-        <is>
-          <t>Decisão líquida 10:1</t>
-        </is>
-      </c>
-      <c r="N2" s="23" t="inlineStr">
-        <is>
-          <t>Decisão líquida 20:1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Árvores impulsionadas</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="n">
-        <v>0.2295344679757571</v>
-      </c>
-      <c r="D3" s="24" t="n">
-        <v>0.02506581222288731</v>
-      </c>
-      <c r="E3" s="24" t="n">
-        <v>1.086640234786473</v>
-      </c>
-      <c r="F3" s="24" t="n">
-        <v>-0.02831372516967114</v>
-      </c>
-      <c r="G3" s="24" t="n">
-        <v>0.785234899328859</v>
-      </c>
-      <c r="H3" s="24" t="n">
-        <v>0.8462323871758219</v>
-      </c>
-      <c r="I3" s="24" t="n">
-        <v>0.1344827586206896</v>
-      </c>
-      <c r="J3" s="24" t="n">
-        <v>0.9923371647509579</v>
-      </c>
-      <c r="K3" s="24" t="n">
-        <v>0.1724137931034483</v>
-      </c>
-      <c r="L3" s="24" t="n">
-        <v>0.006024573919936584</v>
-      </c>
-      <c r="M3" s="24" t="n">
-        <v>0.01080063416567578</v>
-      </c>
-      <c r="N3" s="24" t="n">
-        <v>0.01603250099088387</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Cobertura de juros</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="n">
-        <v>0.1844374990629637</v>
-      </c>
-      <c r="D4" s="24" t="n">
-        <v>0.02561585837572898</v>
-      </c>
-      <c r="E4" s="24" t="n">
-        <v>0.9879690002439582</v>
-      </c>
-      <c r="F4" s="24" t="n">
-        <v>-0.004322604940026632</v>
-      </c>
-      <c r="G4" s="24" t="n">
-        <v>0.785234899328859</v>
-      </c>
-      <c r="H4" s="24" t="n">
-        <v>0.8311210945476822</v>
-      </c>
-      <c r="I4" s="24" t="n">
-        <v>0.1239406779661017</v>
-      </c>
-      <c r="J4" s="24" t="n">
-        <v>0.9921989273525109</v>
-      </c>
-      <c r="K4" s="24" t="n">
-        <v>0.1870788743559255</v>
-      </c>
-      <c r="L4" s="24" t="n">
-        <v>0.002695204122076893</v>
-      </c>
-      <c r="M4" s="24" t="n">
-        <v>0.009274673008323424</v>
-      </c>
-      <c r="N4" s="24" t="n">
-        <v>0.01489298454221165</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Retorno sobre ativos</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="n">
-        <v>0.1753661270949595</v>
-      </c>
-      <c r="D5" s="24" t="n">
-        <v>0.02597582725174593</v>
-      </c>
-      <c r="E5" s="24" t="n">
-        <v>0.9931475518719396</v>
-      </c>
-      <c r="F5" s="24" t="n">
-        <v>-0.004774228210969339</v>
-      </c>
-      <c r="G5" s="24" t="n">
-        <v>0.7919463087248322</v>
-      </c>
-      <c r="H5" s="24" t="n">
-        <v>0.8427608740044925</v>
-      </c>
-      <c r="I5" s="24" t="n">
-        <v>0.1328828828828829</v>
-      </c>
-      <c r="J5" s="24" t="n">
-        <v>0.9925444925444925</v>
-      </c>
-      <c r="K5" s="24" t="n">
-        <v>0.1759809750297265</v>
-      </c>
-      <c r="L5" s="24" t="n">
-        <v>0.002695204122076893</v>
-      </c>
-      <c r="M5" s="24" t="n">
-        <v>0.008997225525168448</v>
-      </c>
-      <c r="N5" s="24" t="n">
-        <v>0.01546769718588981</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Mínimos quadrados parciais</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="n">
-        <v>0.1719750799692672</v>
-      </c>
-      <c r="D6" s="24" t="n">
-        <v>0.02603112214350956</v>
-      </c>
-      <c r="E6" s="24" t="n">
-        <v>1.07206022415256</v>
-      </c>
-      <c r="F6" s="24" t="n">
-        <v>0.007250948427309378</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>0.7919463087248322</v>
-      </c>
-      <c r="H6" s="24" t="n">
-        <v>0.8100878088625689</v>
-      </c>
-      <c r="I6" s="24" t="n">
-        <v>0.1125954198473282</v>
-      </c>
-      <c r="J6" s="24" t="n">
-        <v>0.9922461230615308</v>
-      </c>
-      <c r="K6" s="24" t="n">
-        <v>0.2076892588188664</v>
-      </c>
-      <c r="L6" s="24" t="n">
-        <v>0.002338485929449069</v>
-      </c>
-      <c r="M6" s="24" t="n">
-        <v>0.008085612366230677</v>
-      </c>
-      <c r="N6" s="24" t="n">
-        <v>0.01439754260800634</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Componentes principais (F)</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="n">
-        <v>0.1112965384710407</v>
-      </c>
-      <c r="D7" s="24" t="n">
-        <v>0.02752650275823896</v>
-      </c>
-      <c r="E7" s="24" t="n">
-        <v>0.9913595502153402</v>
-      </c>
-      <c r="F7" s="24" t="n">
-        <v>-0.005980251387520434</v>
-      </c>
-      <c r="G7" s="24" t="n">
-        <v>0.7986577181208053</v>
-      </c>
-      <c r="H7" s="24" t="n">
-        <v>0.5699407800694303</v>
-      </c>
-      <c r="I7" s="24" t="n">
-        <v>0.05348314606741573</v>
-      </c>
-      <c r="J7" s="24" t="n">
-        <v>0.989365473236441</v>
-      </c>
-      <c r="K7" s="24" t="n">
-        <v>0.4409433214427269</v>
-      </c>
-      <c r="L7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="24" t="n">
-        <v>0.003032104637336504</v>
-      </c>
-      <c r="N7" s="24" t="n">
-        <v>0.008531510107015458</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Brito e Assaf Neto</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="n">
-        <v>0.09476579481990252</v>
-      </c>
-      <c r="D8" s="24" t="n">
-        <v>0.02777774711172786</v>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>1.075469920058045</v>
-      </c>
-      <c r="F8" s="24" t="n">
-        <v>0.01462486734399807</v>
-      </c>
-      <c r="G8" s="24" t="n">
-        <v>0.8187919463087249</v>
-      </c>
-      <c r="H8" s="24" t="n">
-        <v>0.4617112517868083</v>
-      </c>
-      <c r="I8" s="24" t="n">
-        <v>0.04423495286439449</v>
-      </c>
-      <c r="J8" s="24" t="n">
-        <v>0.9881993006993007</v>
-      </c>
-      <c r="K8" s="24" t="n">
-        <v>0.5465715418152992</v>
-      </c>
-      <c r="L8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="24" t="n">
-        <v>0.001149425287356322</v>
-      </c>
-      <c r="N8" s="24" t="n">
-        <v>0.009373761395164486</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1 ano</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Referência sem informação</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="n">
-        <v>0.02952833927863655</v>
-      </c>
-      <c r="D9" s="24" t="n">
-        <v>0.02865641645808228</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Árvores impulsionadas</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="n">
-        <v>0.08521677951450135</v>
-      </c>
-      <c r="D10" s="24" t="n">
-        <v>0.02766025850960952</v>
-      </c>
-      <c r="E10" s="24" t="n">
-        <v>1.158922573673336</v>
-      </c>
-      <c r="F10" s="24" t="n">
-        <v>-0.06657935493350987</v>
-      </c>
-      <c r="G10" s="24" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="H10" s="24" t="n">
-        <v>0.4992802303262956</v>
-      </c>
-      <c r="I10" s="24" t="n">
-        <v>0.0479014598540146</v>
-      </c>
-      <c r="J10" s="24" t="n">
-        <v>0.9900095147478591</v>
-      </c>
-      <c r="K10" s="24" t="n">
-        <v>0.5104797391709361</v>
-      </c>
-      <c r="L10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="24" t="n">
-        <v>0.0003493246390312063</v>
-      </c>
-      <c r="N10" s="24" t="n">
-        <v>0.00716115510013973</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Cobertura de juros</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="n">
-        <v>0.05062672744829048</v>
-      </c>
-      <c r="D11" s="24" t="n">
-        <v>0.02815802062181195</v>
-      </c>
-      <c r="E11" s="24" t="n">
-        <v>0.9483481095724542</v>
-      </c>
-      <c r="F11" s="24" t="n">
-        <v>-0.004682623198508686</v>
-      </c>
-      <c r="G11" s="24" t="n">
-        <v>0.8015873015873016</v>
-      </c>
-      <c r="H11" s="24" t="n">
-        <v>0.4517754318618042</v>
-      </c>
-      <c r="I11" s="24" t="n">
-        <v>0.04233025984911987</v>
-      </c>
-      <c r="J11" s="24" t="n">
-        <v>0.9868972746331237</v>
-      </c>
-      <c r="K11" s="24" t="n">
-        <v>0.5556590591523055</v>
-      </c>
-      <c r="L11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="24" t="n">
-        <v>0.003446669771774569</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Retorno sobre ativos</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="n">
-        <v>0.0657719994412717</v>
-      </c>
-      <c r="D12" s="24" t="n">
-        <v>0.02788264124527806</v>
-      </c>
-      <c r="E12" s="24" t="n">
-        <v>0.9751588747917186</v>
-      </c>
-      <c r="F12" s="24" t="n">
-        <v>-0.002241119276739794</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>0.8015873015873016</v>
-      </c>
-      <c r="H12" s="24" t="n">
-        <v>0.5890115163147792</v>
-      </c>
-      <c r="I12" s="24" t="n">
-        <v>0.05567805953693495</v>
-      </c>
-      <c r="J12" s="24" t="n">
-        <v>0.9899193548387096</v>
-      </c>
-      <c r="K12" s="24" t="n">
-        <v>0.4224499301350722</v>
-      </c>
-      <c r="L12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="24" t="n">
-        <v>-0.0006054960409874245</v>
-      </c>
-      <c r="N12" s="24" t="n">
-        <v>0.004413134606427572</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Mínimos quadrados parciais</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="n">
-        <v>0.0644946967358081</v>
-      </c>
-      <c r="D13" s="24" t="n">
-        <v>0.02788026651722164</v>
-      </c>
-      <c r="E13" s="24" t="n">
-        <v>1.075412988199589</v>
-      </c>
-      <c r="F13" s="24" t="n">
-        <v>-0.008215222846687494</v>
-      </c>
-      <c r="G13" s="24" t="n">
-        <v>0.7936507936507936</v>
-      </c>
-      <c r="H13" s="24" t="n">
-        <v>0.5328694817658349</v>
-      </c>
-      <c r="I13" s="24" t="n">
-        <v>0.04885197850512946</v>
-      </c>
-      <c r="J13" s="24" t="n">
-        <v>0.9884290164663997</v>
-      </c>
-      <c r="K13" s="24" t="n">
-        <v>0.4767116907312529</v>
-      </c>
-      <c r="L13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="24" t="n">
-        <v>-0.000232883092687471</v>
-      </c>
-      <c r="N13" s="24" t="n">
-        <v>0.006590591523055425</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Componentes principais (F)</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="n">
-        <v>0.05391257689226329</v>
-      </c>
-      <c r="D14" s="24" t="n">
-        <v>0.02829360358512675</v>
-      </c>
-      <c r="E14" s="24" t="n">
-        <v>0.9153978808503124</v>
-      </c>
-      <c r="F14" s="24" t="n">
-        <v>-0.001851267795798534</v>
-      </c>
-      <c r="G14" s="24" t="n">
-        <v>0.7936507936507936</v>
-      </c>
-      <c r="H14" s="24" t="n">
-        <v>0.2881477927063339</v>
-      </c>
-      <c r="I14" s="24" t="n">
-        <v>0.032605151613955</v>
-      </c>
-      <c r="J14" s="24" t="n">
-        <v>0.9788101059494703</v>
-      </c>
-      <c r="K14" s="24" t="n">
-        <v>0.7142524452724732</v>
-      </c>
-      <c r="L14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="24" t="n">
-        <v>0.003435025617140196</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Brito e Assaf Neto</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="n">
-        <v>0.06037014219553517</v>
-      </c>
-      <c r="D15" s="24" t="n">
-        <v>0.02812598530144687</v>
-      </c>
-      <c r="E15" s="24" t="n">
-        <v>1.260703044771871</v>
-      </c>
-      <c r="F15" s="24" t="n">
-        <v>-0.008544417368427756</v>
-      </c>
-      <c r="G15" s="24" t="n">
-        <v>0.8492063492063492</v>
-      </c>
-      <c r="H15" s="24" t="n">
-        <v>0.2922264875239923</v>
-      </c>
-      <c r="I15" s="24" t="n">
-        <v>0.03500163559044815</v>
-      </c>
-      <c r="J15" s="24" t="n">
-        <v>0.98464025869038</v>
-      </c>
-      <c r="K15" s="24" t="n">
-        <v>0.7119236143455985</v>
-      </c>
-      <c r="L15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="24" t="n">
-        <v>0.004843968327899395</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2 anos</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Referência sem informação</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="n">
-        <v>0.02934326967862133</v>
-      </c>
-      <c r="D16" s="24" t="n">
-        <v>0.02848224220318903</v>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Fonte: script 14. Calibração logística sobre o posto do escore na distribuição do treino; limiar que atinge sensibilidade de 80% nas firmas de treino, aplicado às de teste. Decisão líquida por firma-ano; a de não sinalizar ninguém é zero.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2715,7 +1993,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>0.6266128172318191</v>
+        <v>0.6266128172318192</v>
       </c>
       <c r="C4" s="17" t="n"/>
       <c r="D4" s="17" t="n"/>
@@ -2730,17 +2008,17 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.751919385796545</v>
+        <v>0.7525839350455473</v>
       </c>
       <c r="C5" s="17">
         <f>B5-$B$4</f>
         <v/>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.0597613988902714</v>
+        <v>0.0599783549713972</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.191405616559016</v>
+        <v>0.1922636251348856</v>
       </c>
       <c r="F5" s="16" t="n">
         <v>0.0005</v>
@@ -2757,7 +2035,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.681287702221004</v>
+        <v>0.6812877022210035</v>
       </c>
       <c r="C6" s="17">
         <f>B6-$B$4</f>
@@ -2767,7 +2045,7 @@
         <v>0.008098410066950199</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.105182287672428</v>
+        <v>0.1051822876724277</v>
       </c>
       <c r="F6" s="16" t="n">
         <v>0.02</v>
@@ -2784,7 +2062,7 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.724754745148219</v>
+        <v>0.7247547451482192</v>
       </c>
       <c r="C7" s="17">
         <f>B7-$B$4</f>
@@ -2794,7 +2072,7 @@
         <v>0.0493803501518459</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.147854404332523</v>
+        <v>0.1478544043325228</v>
       </c>
       <c r="F7" s="16" t="n">
         <v>0.0005</v>
@@ -2811,7 +2089,7 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.73071664686348</v>
+        <v>0.7307166468634799</v>
       </c>
       <c r="C8" s="17">
         <f>B8-$B$4</f>
@@ -2821,7 +2099,7 @@
         <v>0.0596128290521198</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.147957724829731</v>
+        <v>0.1479577248297307</v>
       </c>
       <c r="F8" s="16" t="n">
         <v>0.0005</v>
@@ -2865,7 +2143,7 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>0.5680791670474969</v>
+        <v>0.5680791670474972</v>
       </c>
       <c r="C10" s="17">
         <f>B10-$B$4</f>
@@ -2892,14 +2170,14 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>0.505255461109588</v>
+        <v>0.5052554611095877</v>
       </c>
       <c r="C11" s="17">
         <f>B11-$B$4</f>
         <v/>
       </c>
       <c r="D11" s="17" t="n">
-        <v>-0.171218726408485</v>
+        <v>-0.1712187264084851</v>
       </c>
       <c r="E11" s="17" t="n">
         <v>-0.0753579660663876</v>
@@ -2913,18 +2191,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Fonte: 01 e 02. Validação cruzada agrupada por firma, atribuição de referência. Diferença por fórmula. p ajustado por Bonferroni para as seis comparações contra benchmarks e referência não linear; a comparação com mínimos quadrados parciais responde a H4 e não é ajustada.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Fonte: 01 e 02. Validação cruzada agrupada por firma, atribuição de referência. Diferença e p ajustado por fórmula.</t>
-        </is>
-      </c>
+      <c r="A13" s="18" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2992,13 +2266,13 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>0.743835421412301</v>
+        <v>0.7438354214123006</v>
       </c>
       <c r="C4" s="17" t="n"/>
       <c r="D4" s="17" t="n"/>
       <c r="E4" s="17" t="n"/>
       <c r="F4" s="16" t="n">
-        <v>0.680818252759095</v>
+        <v>0.6808182527590948</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -3008,20 +2282,20 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.910136674259681</v>
+        <v>0.9111332574031891</v>
       </c>
       <c r="C5" s="17">
         <f>B5-$B$4</f>
         <v/>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.0767620987579285</v>
+        <v>0.07675753614260297</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.265051116539149</v>
+        <v>0.2647359585531192</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>0.712682546170711</v>
+        <v>0.7084277804615213</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
@@ -3031,20 +2305,20 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.9035449886104781</v>
+        <v>0.9035449886104784</v>
       </c>
       <c r="C6" s="17">
         <f>B6-$B$4</f>
         <v/>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.06683609790819089</v>
+        <v>0.06683609790819094</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>0.25787137641433</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.727249080301735</v>
+        <v>0.7272490803017353</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
@@ -3054,20 +2328,20 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.8995017084282459</v>
+        <v>0.8995017084282461</v>
       </c>
       <c r="C7" s="17">
         <f>B7-$B$4</f>
         <v/>
       </c>
       <c r="D7" s="17" t="n">
-        <v>0.063143941202702</v>
+        <v>0.06314394120270203</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.258642713944733</v>
+        <v>0.2586427139447331</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>0.6897736984876069</v>
+        <v>0.6897736984876073</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
@@ -3077,7 +2351,7 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.890546697038724</v>
+        <v>0.8905466970387244</v>
       </c>
       <c r="C8" s="17">
         <f>B8-$B$4</f>
@@ -3090,7 +2364,7 @@
         <v>0.252442977628922</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>0.722093196090818</v>
+        <v>0.7220931960908179</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="12">
@@ -3100,7 +2374,7 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>0.787015945330296</v>
+        <v>0.7870159453302962</v>
       </c>
       <c r="C9" s="17">
         <f>B9-$B$4</f>
@@ -3109,7 +2383,7 @@
       <c r="D9" s="17" t="n"/>
       <c r="E9" s="17" t="n"/>
       <c r="F9" s="16" t="n">
-        <v>0.686262123295307</v>
+        <v>0.6862621232953068</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
@@ -3132,7 +2406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="11" min="1" max="1"/>
@@ -3182,6 +2456,11 @@
           <t>ROA</t>
         </is>
       </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>MEB</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="12">
       <c r="A4" s="15" t="inlineStr">
@@ -3189,7 +2468,7 @@
           <t>Um ano</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="16" t="n"/>
       <c r="D4" s="16" t="n"/>
       <c r="E4" s="16" t="n"/>
@@ -3202,23 +2481,26 @@
           <t>Somente por EBITDA negativo</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="20" t="n">
         <v>66</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>0.645674841121033</v>
+        <v>0.6456748411210327</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>0.969020303092184</v>
+        <v>0.9691742315951016</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>0.97298748151311</v>
+        <v>0.9729874815131095</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>0.938500999375004</v>
+        <v>0.9385009993750039</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>0.911730125432392</v>
+        <v>0.9117301254323922</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.978129776424651</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
@@ -3227,23 +2509,26 @@
           <t>Patrimônio líquido negativo</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="20" t="n">
         <v>70</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.858013360949853</v>
+        <v>0.8580133609498526</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.836109571457744</v>
+        <v>0.83640085766796</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.8251101257329559</v>
+        <v>0.8251101257329561</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.806182502406721</v>
+        <v>0.8061825024067213</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>0.833224423116194</v>
+        <v>0.8332244231161937</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.6893593745441817</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
@@ -3252,17 +2537,17 @@
           <t>Recuperação judicial</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="20" t="n">
         <v>20</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>0.887505615683071</v>
+        <v>0.8875056156830713</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>0.887425975086788</v>
+        <v>0.8865489074943843</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>0.869802940575863</v>
+        <v>0.8698029405758628</v>
       </c>
       <c r="F7" s="16" t="n">
         <v>0.922327955891362</v>
@@ -3270,6 +2555,9 @@
       <c r="G7" s="16" t="n">
         <v>0.917623034510925</v>
       </c>
+      <c r="H7" t="n">
+        <v>0.779630385950582</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
       <c r="A8" s="15" t="inlineStr">
@@ -3277,23 +2565,26 @@
           <t>Todas as entradas</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>149</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.763207716544714</v>
+        <v>0.7632077165447135</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>0.897094783410745</v>
+        <v>0.8972632196400208</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>0.893687136214063</v>
+        <v>0.8936871362140634</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>0.873822625275302</v>
+        <v>0.8738226252753021</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>0.873875664185579</v>
+        <v>0.8738756641855787</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8242246656972562</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="12">
@@ -3302,7 +2593,7 @@
           <t>Dois anos</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="16" t="n"/>
       <c r="D9" s="16" t="n"/>
       <c r="E9" s="16" t="n"/>
@@ -3315,23 +2606,26 @@
           <t>Somente por EBITDA negativo</t>
         </is>
       </c>
-      <c r="B10" s="19" t="n">
+      <c r="B10" s="20" t="n">
         <v>52</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.37722528790787</v>
+        <v>0.3772252879078695</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.7225567049313451</v>
+        <v>0.7194460080466559</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.522132917466411</v>
+        <v>0.5221329174664107</v>
       </c>
       <c r="F10" s="16" t="n">
         <v>0.649544607264137</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>0.595111102908608</v>
+        <v>0.5951111029086078</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.61837673482947</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
@@ -3340,24 +2634,27 @@
           <t>Patrimônio líquido negativo</t>
         </is>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="20" t="n">
         <v>63</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>0.806624165981172</v>
+        <v>0.8066241659811716</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>0.772177855467203</v>
+        <v>0.771337362520184</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>0.801733921335649</v>
+        <v>0.8017339213356488</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>0.764780413124943</v>
+        <v>0.7647804131249429</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>0.829193705633245</v>
       </c>
+      <c r="H11" t="n">
+        <v>0.6779297291533376</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="12">
       <c r="A12" s="15" t="inlineStr">
@@ -3365,23 +2662,26 @@
           <t>Recuperação judicial</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="20" t="n">
         <v>17</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.806510387264311</v>
+        <v>0.8065103872643107</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.849143332956983</v>
+        <v>0.8503951676639947</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.766484136840917</v>
+        <v>0.7664841368409168</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.859347126566558</v>
+        <v>0.8593471265665575</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>0.825985096533815</v>
+        <v>0.8259850965338151</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.724398780625494</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
@@ -3390,29 +2690,32 @@
           <t>Todas as entradas</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="20" t="n">
         <v>126</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>0.626757151997075</v>
+        <v>0.6267571519970752</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>0.757206075008378</v>
+        <v>0.7554207415531792</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>0.681287702221004</v>
+        <v>0.6812877022210035</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>0.72646638789873</v>
+        <v>0.7264663878987296</v>
       </c>
       <c r="G13" s="16" t="n">
         <v>0.73071664686348</v>
       </c>
+      <c r="H13" t="n">
+        <v>0.6538250616945434</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="12">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Fonte: 09. Médias sobre dez atribuições. Em cada linha, os não eventos são todos os da amostra e os eventos apenas os do tipo indicado.</t>
+          <t>Fonte: 09. Médias sobre dez atribuições. Em cada linha, os não eventos são todos os da amostra e os eventos apenas os do tipo indicado. MEB: margem EBITDA isolada, cuja condição define o critério de prejuízo operacional.</t>
         </is>
       </c>
     </row>
@@ -3476,16 +2779,16 @@
           <t>ROA</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.780783062873292</v>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="21" t="n">
         <v>0.48627472863789</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.889077026811682</v>
       </c>
-      <c r="E4" s="21" t="n">
+      <c r="E4" s="22" t="n">
         <v>0.452236234964863</v>
       </c>
     </row>
@@ -3495,35 +2798,35 @@
           <t>COB</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="21" t="n">
         <v>0.774695135092589</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="21" t="n">
         <v>0.238113071125549</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="21" t="n">
         <v>0.168890555847401</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="22" t="n">
         <v>0.366110304900671</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
+          <t>MEB</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
         <v>0.68833033169227</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="21" t="n">
         <v>0.226029228081107</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.301210882140014</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="22" t="n">
         <v>0.44151965006269</v>
       </c>
     </row>
@@ -3533,16 +2836,16 @@
           <t>CG</t>
         </is>
       </c>
-      <c r="B7" s="20" t="n">
+      <c r="B7" s="21" t="n">
         <v>0.350637278695345</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="21" t="n">
         <v>0.531605179440876</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="21" t="n">
         <v>0.106855974215405</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="22" t="n">
         <v>0.608172927280216</v>
       </c>
     </row>
@@ -3552,16 +2855,16 @@
           <t>LC</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="21" t="n">
         <v>0.342364181207915</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="21" t="n">
         <v>0.373227621659178</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="21" t="n">
         <v>0.195024162423581</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="22" t="n">
         <v>0.55753687407719</v>
       </c>
     </row>
@@ -3571,16 +2874,16 @@
           <t>FCO</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="21" t="n">
         <v>0.323418235110018</v>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="21" t="n">
         <v>0.178921799723756</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="21" t="n">
         <v>0.00650744486255841</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="22" t="n">
         <v>0.287004851493431</v>
       </c>
     </row>
@@ -3590,16 +2893,16 @@
           <t>CP</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <v>0.30599872188187</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="21" t="n">
         <v>0.17114287593687</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="21" t="n">
         <v>0.20193913561241</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="22" t="n">
         <v>0.551880562359334</v>
       </c>
     </row>
@@ -3609,16 +2912,16 @@
           <t>ALV</t>
         </is>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="21" t="n">
         <v>0.176199453894981</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="21" t="n">
         <v>0.415384187135599</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="21" t="n">
         <v>0.00395481183124808</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="22" t="n">
         <v>0.682760454855237</v>
       </c>
     </row>
@@ -3638,241 +2941,716 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" style="11" min="1" max="1"/>
-    <col width="15" customWidth="1" style="11" min="2" max="7"/>
+    <col width="28" customWidth="1" style="12" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="12">
-      <c r="A1" s="13" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Tabela 17 – Métricas de probabilidade e desempenho operacional</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="12">
-      <c r="A3" s="14" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Horizonte</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>AUC precisão-revocação</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>Brier</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>Inclinação</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>Firmas sinalizadas</t>
-        </is>
-      </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Intercepto</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>Sensibilidade</t>
+        </is>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>Especificidade</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
         <is>
           <t>VPP</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>VPN</t>
+        </is>
+      </c>
+      <c r="K3" s="19" t="inlineStr">
+        <is>
+          <t>Firma-anos sinalizados</t>
+        </is>
+      </c>
+      <c r="L3" s="19" t="inlineStr">
+        <is>
+          <t>Decisão líquida 5:1</t>
+        </is>
+      </c>
+      <c r="M3" s="19" t="inlineStr">
         <is>
           <t>Decisão líquida 10:1</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="12">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="N3" s="19" t="inlineStr">
+        <is>
+          <t>Decisão líquida 20:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Árvores impulsionadas</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
-        <v>0.234261627665135</v>
-      </c>
-      <c r="C4" s="16" t="n">
-        <v>0.0265137176514983</v>
-      </c>
-      <c r="D4" s="20" t="n">
-        <v>1.01596915198933</v>
-      </c>
-      <c r="E4" s="21" t="n">
-        <v>0.172017439556084</v>
-      </c>
-      <c r="F4" s="20" t="n">
-        <v>0.13594470046083</v>
-      </c>
-      <c r="G4" s="17" t="n">
-        <v>0.008244153785176379</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="12">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="C4" t="n">
+        <v>0.2295344679757571</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.02506581222288731</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.086640234786473</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.02831372516967114</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.785234899328859</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.8462323871758219</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1344827586206896</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9923371647509579</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1724137931034483</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.006024573919936584</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.01080063416567578</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.01603250099088387</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Cobertura de juros</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
-        <v>0.214733717263813</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>0.0279884457179383</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.970449809886877</v>
-      </c>
-      <c r="E5" s="21" t="n">
-        <v>0.186682520808561</v>
-      </c>
-      <c r="F5" s="20" t="n">
-        <v>0.124203821656051</v>
-      </c>
-      <c r="G5" s="17" t="n">
-        <v>0.00231866825208086</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="12">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="C5" t="n">
+        <v>0.1844374990629637</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.02561585837572898</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9879690002439582</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.004322604940026632</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.785234899328859</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.8311210945476822</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.1239406779661017</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.9921989273525109</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1870788743559255</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.002695204122076893</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.009274673008323424</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.01489298454221165</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Retorno sobre ativos</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.1753661270949595</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.02597582725174593</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9931475518719396</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.004774228210969339</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.7919463087248322</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.8427608740044925</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.1328828828828829</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.9925444925444925</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1759809750297265</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.002695204122076893</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.008997225525168448</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.01546769718588981</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mínimos quadrados parciais</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
-        <v>0.171928329526102</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>0.0288484234983213</v>
-      </c>
-      <c r="D6" s="20" t="n">
-        <v>1.00500507911664</v>
-      </c>
-      <c r="E6" s="21" t="n">
-        <v>0.207689258818866</v>
-      </c>
-      <c r="F6" s="20" t="n">
-        <v>0.112595419847328</v>
-      </c>
-      <c r="G6" s="17" t="n">
-        <v>0.00370590566785573</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="12">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="C7" t="n">
+        <v>0.1719750799692672</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.02603112214350956</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.07206022415256</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.007250948427309378</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.7919463087248322</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.8100878088625689</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.1125954198473282</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9922461230615308</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.2076892588188664</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.002338485929449069</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.008085612366230677</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.01439754260800634</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Componentes principais (F)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.1112965384710407</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.02752650275823896</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9913595502153402</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.005980251387520434</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.7986577181208053</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.5699407800694303</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.05348314606741573</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.989365473236441</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.4409433214427269</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.003032104637336504</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.008531510107015458</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Brito e Assaf Neto</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.09476579481990252</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.02777774711172786</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.075469920058045</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.01462486734399807</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.8187919463087249</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.4617112517868083</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.04423495286439449</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.9881993006993007</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.5465715418152992</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.001149425287356322</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.009373761395164486</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>um ano</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Referência sem informação</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.02952833927863655</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.02865641645808228</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Árvores impulsionadas</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.08521677951450135</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.02766025850960952</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.158922573673336</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.06657935493350987</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.4992802303262956</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0479014598540146</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.9900095147478591</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.5104797391709361</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.0003493246390312063</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.00716115510013973</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cobertura de juros</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.05062672744829048</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.02815802062181195</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.9483481095724542</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.004682623198508686</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.8015873015873016</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.4517754318618042</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.04233025984911987</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.9868972746331237</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.5556590591523055</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.003446669771774569</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Retorno sobre ativos</t>
         </is>
       </c>
-      <c r="B7" s="20" t="n">
-        <v>0.17144107679132</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>0.0289235936489408</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <v>0.9681216349381651</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>0.175782798256044</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>0.133032694475761</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <v>0.00307173999207293</v>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="12">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="C13" t="n">
+        <v>0.0657719994412717</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.02788264124527806</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.9751588747917186</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-0.002241119276739794</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.8015873015873016</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.5890115163147792</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.05567805953693495</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.9899193548387096</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.4224499301350722</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>-0.0006054960409874245</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.004413134606427572</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mínimos quadrados parciais</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0644946967358081</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.02788026651722164</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.075412988199589</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.008215222846687494</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.7936507936507936</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.5328694817658349</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.04885197850512946</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.9884290164663997</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.4767116907312529</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-0.000232883092687471</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.006590591523055425</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Componentes principais (F)</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
-        <v>0.109522282672632</v>
-      </c>
-      <c r="C8" s="16" t="n">
-        <v>0.0285132844958893</v>
-      </c>
-      <c r="D8" s="20" t="n">
-        <v>0.973015511320882</v>
-      </c>
-      <c r="E8" s="21" t="n">
-        <v>0.440943321442727</v>
-      </c>
-      <c r="F8" s="20" t="n">
-        <v>0.0534831460674157</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>0.00124851367419738</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="12">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="C15" t="n">
+        <v>0.05391257689226329</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.02829360358512675</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.9153978808503124</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.001851267795798534</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.7936507936507936</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.2881477927063339</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.032605151613955</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.9788101059494703</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.7142524452724732</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.003435025617140196</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Brito e Assaf Neto</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n">
-        <v>0.07676792535361621</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>0.0290237015411308</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0.738041435678831</v>
-      </c>
-      <c r="E9" s="21" t="n">
-        <v>0.545977011494253</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>0.0442831215970962</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>-5.94530321046373e-05</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="12">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="C16" t="n">
+        <v>0.06037014219553517</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.02812598530144687</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.260703044771871</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.008544417368427756</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.8492063492063492</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.2922264875239923</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.03500163559044815</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.98464025869038</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.7119236143455985</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.004843968327899395</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>dois anos</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Referência sem informação</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
-        <v>0.0295283392786366</v>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>0.0286564164580823</v>
-      </c>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="17" t="n">
-        <v>-0.0675188267934998</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Fonte: 03. Limiar que atinge sensibilidade de 80% nas firmas de treino, aplicado às de teste.</t>
+      <c r="C17" t="n">
+        <v>0.02934326967862133</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.02848224220318903</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Fonte: 14. Calibração logística sobre o posto do escore na distribuição do treino; limiar que atinge sensibilidade de 80% nas firmas de treino, aplicado às de teste. Decisão líquida por firma-ano; a de não sinalizar ninguém é zero.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -3939,23 +3717,23 @@
           <t>Definição principal</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n">
+      <c r="B4" s="23" t="n">
         <v>5046</v>
       </c>
-      <c r="C4" s="19" t="n">
+      <c r="C4" s="20" t="n">
         <v>149</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>0.763207716544714</v>
+        <v>0.7632077165447135</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>0.897094783410745</v>
+        <v>0.8972632196400208</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>0.893687136214063</v>
+        <v>0.8936871362140634</v>
       </c>
       <c r="G4" s="16" t="n">
-        <v>0.873822625275302</v>
+        <v>0.8738226252753021</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -3964,20 +3742,20 @@
           <t>Sem as entradas exclusivas do critério de EBITDA</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>4980</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <v>83</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>0.856667593387641</v>
+        <v>0.8566675933876409</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>0.85752083276951</v>
+        <v>0.8571074988128951</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>0.830629030313617</v>
+        <v>0.8306290303136171</v>
       </c>
       <c r="G5" s="16" t="n">
         <v>0.856184632341906</v>
@@ -3989,23 +3767,23 @@
           <t>Restritiva: PL negativo ou recuperação judicial</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <v>5575</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="20" t="n">
         <v>81</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.889054726368159</v>
+        <v>0.8890547263681592</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.9546189558081321</v>
+        <v>0.9541473976099629</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.900035729213014</v>
+        <v>0.9000357292130137</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>0.931884165441986</v>
+        <v>0.9318841654419862</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
@@ -4028,7 +3806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="11" min="1" max="1"/>
@@ -4090,23 +3868,23 @@
           <t>Especificação principal</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n">
+      <c r="B4" s="23" t="n">
         <v>5046</v>
       </c>
-      <c r="C4" s="19" t="n">
+      <c r="C4" s="20" t="n">
         <v>149</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>0.764267398338662</v>
+        <v>0.7642673983386623</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>0.875253031235395</v>
+        <v>0.8752530312353954</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>0.893687136214063</v>
+        <v>0.8936871362140634</v>
       </c>
       <c r="G4" s="16" t="n">
-        <v>0.873875664185579</v>
+        <v>0.8738756641855786</v>
       </c>
       <c r="H4" s="17">
         <f>E4-D4</f>
@@ -4119,20 +3897,20 @@
           <t>Excluídas as entradas exclusivamente por recuperação judicial</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>5035</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <v>138</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>0.759206316792594</v>
+        <v>0.7592063167925941</v>
       </c>
       <c r="E5" s="16" t="n">
         <v>0.875920779655098</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>0.898019491377448</v>
+        <v>0.8980194913774479</v>
       </c>
       <c r="G5" s="16" t="n">
         <v>0.873017493703628</v>
@@ -4148,23 +3926,23 @@
           <t>Somente a primeira entrada de cada firma</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <v>4629</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="20" t="n">
         <v>130</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.789324123309453</v>
+        <v>0.7893241233094533</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.897084822268196</v>
+        <v>0.8970848222681963</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.90651426812796</v>
+        <v>0.9065142681279601</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>0.886800485577992</v>
+        <v>0.8868004855779917</v>
       </c>
       <c r="H6" s="17">
         <f>E6-D6</f>
@@ -4177,23 +3955,23 @@
           <t>Saídas associadas a distress tratadas como evento</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
-        <v>5052</v>
-      </c>
-      <c r="C7" s="19" t="n">
-        <v>155</v>
+      <c r="B7" s="23" t="n">
+        <v>5055</v>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>158</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>0.7665311876263941</v>
+        <v>0.7705428019738254</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>0.877987181091781</v>
+        <v>0.8796395623256812</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>0.894770992114988</v>
+        <v>0.8962235985348819</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>0.875601256859038</v>
+        <v>0.876524764580743</v>
       </c>
       <c r="H7" s="17">
         <f>E7-D7</f>
@@ -4201,36 +3979,66 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saídas por dificuldade financeira segundo o cadastro, como evento</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5057</v>
+      </c>
+      <c r="C8" t="n">
+        <v>160</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.7618031447825199</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.8717365223606289</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8885829334286298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.8708890647335104</v>
+      </c>
+      <c r="H8">
+        <f>E8-D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Somente firmas com registro ativo ao fim do período</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>4201</v>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C9" s="20" t="n">
         <v>104</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D9" s="16" t="n">
         <v>0.744979910253281</v>
       </c>
-      <c r="E8" s="16" t="n">
-        <v>0.890046187641989</v>
-      </c>
-      <c r="F8" s="16" t="n">
-        <v>0.90976629240908</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>0.892249957755206</v>
-      </c>
-      <c r="H8" s="17">
-        <f>E8-D8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="12">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="E9" s="16" t="n">
+        <v>0.8900461876419894</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>0.9097662924090798</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>0.8922499577552055</v>
+      </c>
+      <c r="H9" s="17">
+        <f>E9-D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="12"/>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Fonte: 04, 05 e 07. Horizonte de um ano, atribuição de referência.</t>
         </is>
@@ -4287,7 +4095,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>0.762685824631709</v>
+        <v>0.7626858246317085</v>
       </c>
       <c r="C4" s="17" t="n"/>
     </row>
@@ -4298,7 +4106,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.778659170866151</v>
+        <v>0.7786591708661514</v>
       </c>
       <c r="C5" s="17">
         <f>B5-B4</f>
@@ -4312,7 +4120,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.886041035944483</v>
+        <v>0.8860410359444832</v>
       </c>
       <c r="C6" s="17" t="n"/>
     </row>
@@ -4323,7 +4131,7 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>0.885591507195886</v>
+        <v>0.8855915071958863</v>
       </c>
       <c r="C7" s="17">
         <f>B7-B6</f>
@@ -4337,7 +4145,7 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>0.875983515451866</v>
+        <v>0.8759835154518655</v>
       </c>
       <c r="C8" s="17" t="n"/>
     </row>
@@ -4348,7 +4156,7 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>0.853337134226818</v>
+        <v>0.8533371342268175</v>
       </c>
       <c r="C9" s="17">
         <f>B9-B8</f>

</xml_diff>

<commit_message>
Correcao do painel (3 emissores estrangeiros e 4 firma-anos) com particoes preservadas; nova execucao; v4 com numeros, tabelas e figuras atualizados; segunda leva de citacoes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4LwoZDLWB9PeJtPghPCix
</commit_message>
<xml_diff>
--- a/projeto/tabelas/Tabelas_Artigo_revisado.xlsx
+++ b/projeto/tabelas/Tabelas_Artigo_revisado.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="11" min="1" max="1"/>
@@ -463,7 +463,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Numeração das tabelas: abas desta planilha e versão final do artigo (com o Apêndice A)</t>
+          <t>Numeração das tabelas: abas desta planilha e versão 4 do artigo (com a Tabela 1 do panorama e o Apêndice A)</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -505,7 +505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -535,7 +535,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -781,6 +781,13 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>Apêndice A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>A Tabela 1 da versão 4 (panorama, seção 2) não tem aba: é gerada pelo script 17_panorama.py.</t>
         </is>
       </c>
     </row>
@@ -833,7 +840,7 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>0.7626858246317085</v>
+        <v>0.761799887960105</v>
       </c>
       <c r="C4" s="18" t="n"/>
     </row>
@@ -844,7 +851,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>0.7786591708661514</v>
+        <v>0.779085062445765</v>
       </c>
       <c r="C5" s="18">
         <f>B5-B4</f>
@@ -858,7 +865,7 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>0.8860410359444832</v>
+        <v>0.8865767692966751</v>
       </c>
       <c r="C6" s="18" t="n"/>
     </row>
@@ -869,7 +876,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>0.8855915071958863</v>
+        <v>0.8860742374147343</v>
       </c>
       <c r="C7" s="18">
         <f>B7-B6</f>
@@ -883,7 +890,7 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>0.8759835154518655</v>
+        <v>0.8763579345115829</v>
       </c>
       <c r="C8" s="18" t="n"/>
     </row>
@@ -894,7 +901,7 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>0.8533371342268175</v>
+        <v>0.853306000724964</v>
       </c>
       <c r="C9" s="18">
         <f>B9-B8</f>
@@ -974,16 +981,16 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>0.7642673983386623</v>
+        <v>0.76321274398884</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>0.8752530312353954</v>
+        <v>0.8767190434868573</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>0.8969839087895205</v>
+        <v>0.8968917167367831</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>0.7344984533744122</v>
+        <v>0.7352233658102572</v>
       </c>
       <c r="F4" s="18">
         <f>C4-B4</f>
@@ -997,16 +1004,16 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>0.7646511423923427</v>
+        <v>0.7635587495468975</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>0.8747240126471076</v>
+        <v>0.8751167082239479</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.8904170886709162</v>
+        <v>0.8919934039257901</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.7391102345909631</v>
+        <v>0.7397159459132899</v>
       </c>
       <c r="F5" s="18">
         <f>C5-B5</f>
@@ -1020,16 +1027,16 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>0.7612125215684716</v>
+        <v>0.760230505607487</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>0.8741922530298649</v>
+        <v>0.875020595568932</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.905770962361561</v>
+        <v>0.9054443699952768</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.7334280815675397</v>
+        <v>0.7341125781258582</v>
       </c>
       <c r="F6" s="18">
         <f>C6-B6</f>
@@ -1043,16 +1050,16 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>0.7621801047895369</v>
+        <v>0.7611820208921452</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>0.877347177356908</v>
+        <v>0.8775675809268555</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>0.8955866692797809</v>
+        <v>0.8951465855292786</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.7336076189640829</v>
+        <v>0.7339807664846933</v>
       </c>
       <c r="F7" s="18">
         <f>C7-B7</f>
@@ -1066,16 +1073,16 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>0.7652185353859986</v>
+        <v>0.7642809674974461</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>0.8687088246056687</v>
+        <v>0.8681581520007908</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>0.8922378171541815</v>
+        <v>0.8913453300233966</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.7054654746845418</v>
+        <v>0.7058115203374378</v>
       </c>
       <c r="F8" s="18">
         <f>C8-B8</f>
@@ -1089,16 +1096,16 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>0.7625940001617207</v>
+        <v>0.7616159008776459</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>0.8750885694981039</v>
+        <v>0.8749025143070552</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>0.9002519005609516</v>
+        <v>0.8970331396434496</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>0.7277130361966578</v>
+        <v>0.7282332297147377</v>
       </c>
       <c r="F9" s="18">
         <f>C9-B9</f>
@@ -1112,16 +1119,16 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>0.7602668665790451</v>
+        <v>0.7591773855160975</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>0.8700861916554855</v>
+        <v>0.8702698843352848</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>0.8994330181606873</v>
+        <v>0.8980697832796933</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>0.7252241819056455</v>
+        <v>0.7258111908083349</v>
       </c>
       <c r="F10" s="18">
         <f>C10-B10</f>
@@ -1135,16 +1142,16 @@
         </is>
       </c>
       <c r="B11" s="17" t="n">
-        <v>0.7638192401045428</v>
+        <v>0.7627802370412681</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>0.8754024173134353</v>
+        <v>0.8759968255363086</v>
       </c>
       <c r="D11" s="17" t="n">
-        <v>0.8989204457461286</v>
+        <v>0.8996982062632498</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>0.7316340781165842</v>
+        <v>0.7324223684355057</v>
       </c>
       <c r="F11" s="18">
         <f>C11-B11</f>
@@ -1158,16 +1165,16 @@
         </is>
       </c>
       <c r="B12" s="17" t="n">
-        <v>0.7648745362521637</v>
+        <v>0.763870429156735</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>0.876013666770369</v>
+        <v>0.876330473753007</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>0.8942250631464546</v>
+        <v>0.8963596645393732</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>0.7059204854910485</v>
+        <v>0.7064541020881161</v>
       </c>
       <c r="F12" s="18">
         <f>C12-B12</f>
@@ -1181,16 +1188,16 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>0.7629928198746527</v>
+        <v>0.7621390283285185</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>0.8714101086406826</v>
+        <v>0.8717060820088094</v>
       </c>
       <c r="D13" s="17" t="n">
-        <v>0.8988053225300245</v>
+        <v>0.9017014686013687</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>0.7175301136293554</v>
+        <v>0.7182388866310043</v>
       </c>
       <c r="F13" s="18">
         <f>C13-B13</f>
@@ -1351,16 +1358,16 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>0.6266128172318192</v>
+        <v>0.6263262473017398</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>0.7247547451482192</v>
+        <v>0.723652395444803</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>0.7525839350455473</v>
+        <v>0.7486232199110623</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>0.667237912439448</v>
+        <v>0.6683218538096001</v>
       </c>
       <c r="F4" s="18">
         <f>C4-B4</f>
@@ -1374,16 +1381,16 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>0.6269955518995826</v>
+        <v>0.6267686475519249</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>0.720032446759894</v>
+        <v>0.72058801095322</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.7710380297352466</v>
+        <v>0.7683700983196418</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.6679157907564818</v>
+        <v>0.6686975126427313</v>
       </c>
       <c r="F5" s="18">
         <f>C5-B5</f>
@@ -1397,16 +1404,16 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>0.6257235779788562</v>
+        <v>0.6255367916828753</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>0.7374383054565397</v>
+        <v>0.7372943410905929</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.7616648386801937</v>
+        <v>0.7613498546944006</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.6671065259117083</v>
+        <v>0.6679976812124818</v>
       </c>
       <c r="F6" s="18">
         <f>C6-B6</f>
@@ -1420,16 +1427,16 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>0.6262548365475429</v>
+        <v>0.6260669092240452</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>0.7258286872010481</v>
+        <v>0.7242606957888073</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>0.7624036498796576</v>
+        <v>0.7573367886318391</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.677398470584651</v>
+        <v>0.6777323936141812</v>
       </c>
       <c r="F7" s="18">
         <f>C7-B7</f>
@@ -1443,16 +1450,16 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>0.6276353471650976</v>
+        <v>0.6274761065726947</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>0.7234389757182463</v>
+        <v>0.7289287811873107</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>0.7543909758401122</v>
+        <v>0.7557130652998024</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.6658155104652226</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F8" s="18">
         <f>C8-B8</f>
@@ -1466,16 +1473,16 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>0.6266623251987935</v>
+        <v>0.6263853611282731</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>0.7237950522499467</v>
+        <v>0.7277274356803429</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>0.747254211985498</v>
+        <v>0.7468498051150622</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>0.6692391767967584</v>
+        <v>0.6699102995354798</v>
       </c>
       <c r="F9" s="18">
         <f>C9-B9</f>
@@ -1489,16 +1496,16 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>0.6268356030832039</v>
+        <v>0.6266618612846387</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>0.7291019254790848</v>
+        <v>0.7305515510705324</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>0.7652351247600768</v>
+        <v>0.7643932633120524</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>0.6709433933522225</v>
+        <v>0.6714396314348261</v>
       </c>
       <c r="F10" s="18">
         <f>C10-B10</f>
@@ -1512,16 +1519,16 @@
         </is>
       </c>
       <c r="B11" s="17" t="n">
-        <v>0.6266509002833379</v>
+        <v>0.6264387542619162</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>0.7338584986137769</v>
+        <v>0.732511841834283</v>
       </c>
       <c r="D11" s="17" t="n">
-        <v>0.7338708756055206</v>
+        <v>0.7321609726703432</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>0.6637456966151783</v>
+        <v>0.6642525342669504</v>
       </c>
       <c r="F11" s="18">
         <f>C11-B11</f>
@@ -1535,16 +1542,16 @@
         </is>
       </c>
       <c r="B12" s="17" t="n">
-        <v>0.6288521006611217</v>
+        <v>0.6285249002692539</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>0.7228067970630351</v>
+        <v>0.7206681006536845</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>0.7528219541175395</v>
+        <v>0.753242679419998</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>0.6538231575419675</v>
+        <v>0.6545235425581413</v>
       </c>
       <c r="F12" s="18">
         <f>C12-B12</f>
@@ -1558,16 +1565,16 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>0.6253484599213965</v>
+        <v>0.625159225952114</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>0.7236084452975048</v>
+        <v>0.7240776336163169</v>
       </c>
       <c r="D13" s="17" t="n">
-        <v>0.7529438198823996</v>
+        <v>0.755812223976568</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>0.6545943393352223</v>
+        <v>0.6549716635012166</v>
       </c>
       <c r="F13" s="18">
         <f>C13-B13</f>
@@ -1746,25 +1753,25 @@
         <v>66</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>0.6489099696165247</v>
+        <v>0.6468779447502851</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>0.3240775118965847</v>
+        <v>0.3266084536031345</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>0.2441001087008582</v>
+        <v>0.2493054990813685</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>0.4113477358132478</v>
+        <v>0.4097134593232188</v>
       </c>
       <c r="G4" s="18" t="n">
-        <v>0.2906479539111763</v>
+        <v>0.293975970837673</v>
       </c>
       <c r="H4" s="18" t="n">
-        <v>0.2169267391522895</v>
+        <v>0.2229804391120515</v>
       </c>
       <c r="I4" s="18" t="n">
-        <v>0.3713797698784761</v>
+        <v>0.3728411692139859</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
@@ -1777,25 +1784,25 @@
         <v>51</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>0.816061854596852</v>
+        <v>0.8156228940021181</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>-0.02956792273781061</v>
+        <v>-0.02869973685055038</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>-0.09311508603706418</v>
+        <v>-0.09590775513597671</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>0.03786911761045506</v>
+        <v>0.03533681671835408</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>-0.0658906813695459</v>
+        <v>-0.06303552517570044</v>
       </c>
       <c r="H5" s="18" t="n">
-        <v>-0.1288713063873238</v>
+        <v>-0.1284256786414577</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>-0.003360119759590024</v>
+        <v>0.001336722155975431</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
@@ -1808,25 +1815,25 @@
         <v>11</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>0.8277609668257003</v>
+        <v>0.8277600059514953</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.01157480461135763</v>
+        <v>0.0120982740663591</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>-0.09660755535743742</v>
+        <v>-0.08891126902416062</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>0.1166857701718687</v>
+        <v>0.1100396224224637</v>
       </c>
       <c r="G6" s="18" t="n">
-        <v>0.06276570070729759</v>
+        <v>0.06343922035411398</v>
       </c>
       <c r="H6" s="18" t="n">
-        <v>-0.0006642813098388315</v>
+        <v>0.003489187615294262</v>
       </c>
       <c r="I6" s="18" t="n">
-        <v>0.1363261090615032</v>
+        <v>0.1342010797794001</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
@@ -1839,25 +1846,25 @@
         <v>52</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>0.3774961243171416</v>
+        <v>0.3773472442982294</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0.1446367931492692</v>
+        <v>0.1447713747089048</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>0.0572070649833604</v>
+        <v>0.06038623113510876</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>0.2326621229769502</v>
+        <v>0.2301832063857286</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>0.2752473054776318</v>
+        <v>0.2734770635419362</v>
       </c>
       <c r="H7" s="18" t="n">
-        <v>0.1959504804635307</v>
+        <v>0.1923293109904629</v>
       </c>
       <c r="I7" s="18" t="n">
-        <v>0.3530558073446463</v>
+        <v>0.3513485271343187</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
@@ -1870,25 +1877,25 @@
         <v>46</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>0.7955906283902194</v>
+        <v>0.7952071537513319</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>-0.004821935241592246</v>
+        <v>-0.004249106825731763</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0.06892852625382186</v>
+        <v>-0.06783736856145642</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>0.06318414073021726</v>
+        <v>0.0665666337132101</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>-0.08249186347325377</v>
+        <v>-0.08293984915279018</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>-0.1392930511812144</v>
+        <v>-0.1412219039926418</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0.0231236879844152</v>
+        <v>-0.02293671909468541</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
@@ -1901,25 +1908,25 @@
         <v>9</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>0.8008903817445084</v>
+        <v>0.8008970046452026</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>-0.08759863510343358</v>
+        <v>-0.08753804260772069</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>-0.2404160277235961</v>
+        <v>-0.2416744874092348</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>0.06901473373991801</v>
+        <v>0.06564337737752496</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>0.05331627212625289</v>
+        <v>0.05317956110844146</v>
       </c>
       <c r="H9" s="18" t="n">
-        <v>-0.02610726019816766</v>
+        <v>-0.02215458933907346</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>0.1478807596901882</v>
+        <v>0.1466768919158264</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
@@ -1991,7 +1998,7 @@
         <v>0.425126544113893</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>0.326386397196832</v>
+        <v>0.3264330184708675</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
@@ -2007,7 +2014,7 @@
         <v>0.943732022580715</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>1.43043910867033</v>
+        <v>1.428704657601445</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
@@ -2023,7 +2030,7 @@
         <v>-0.024871125548301</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>0.084351266928543</v>
+        <v>0.08432206643525114</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
@@ -2039,7 +2046,7 @@
         <v>0.37655960009212</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>1.50992137747865</v>
+        <v>1.508201100068395</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
@@ -2055,7 +2062,7 @@
         <v>-0.0336808481906868</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>0.0396492206621962</v>
+        <v>0.03963596256557115</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
@@ -2071,7 +2078,7 @@
         <v>0.117722059244612</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>0.211605259184521</v>
+        <v>0.211718870964725</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="11">
@@ -2087,7 +2094,7 @@
         <v>21.4529774714187</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>22.1714420501993</v>
+        <v>22.1732955377026</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
@@ -2103,7 +2110,7 @@
         <v>65</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>4193</v>
+        <v>4186</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="11">
@@ -2184,7 +2191,7 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>0.7642673983386623</v>
+        <v>0.76321274398884</v>
       </c>
       <c r="C4" s="18" t="n"/>
       <c r="D4" s="18" t="n"/>
@@ -2199,17 +2206,17 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>0.8969839087895205</v>
+        <v>0.8968917167367831</v>
       </c>
       <c r="C5" s="18">
         <f>B5-$B$4</f>
         <v/>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.0857751707434312</v>
+        <v>0.0867951986480982</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>0.1813942265915912</v>
+        <v>0.1784190651900804</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>0.0005</v>
@@ -2226,17 +2233,17 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>0.8936871362140634</v>
+        <v>0.8941765342325816</v>
       </c>
       <c r="C6" s="18">
         <f>B6-$B$4</f>
         <v/>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.0800957193667922</v>
+        <v>0.07928160544217169</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>0.1813288756101432</v>
+        <v>0.1773994536971488</v>
       </c>
       <c r="F6" s="17" t="n">
         <v>0.0005</v>
@@ -2253,17 +2260,17 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>0.8752530312353954</v>
+        <v>0.8767190434868573</v>
       </c>
       <c r="C7" s="18">
         <f>B7-$B$4</f>
         <v/>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0.0644198867522225</v>
+        <v>0.0660555626771604</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>0.1603352399513336</v>
+        <v>0.1585463387211497</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>0.0005</v>
@@ -2280,17 +2287,17 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>0.8738756641855786</v>
+        <v>0.8742146223047266</v>
       </c>
       <c r="C8" s="18">
         <f>B8-$B$4</f>
         <v/>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0.0607085903949829</v>
+        <v>0.0637250438088823</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>0.1578004553955183</v>
+        <v>0.1572283507001996</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>0.0005</v>
@@ -2307,20 +2314,20 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>0.7344984533744122</v>
+        <v>0.7352233658102572</v>
       </c>
       <c r="C9" s="18">
         <f>B9-$B$4</f>
         <v/>
       </c>
       <c r="D9" s="18" t="n">
-        <v>-0.0751501393568418</v>
+        <v>-0.0734830669537468</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>0.0162514157036613</v>
+        <v>0.0186818782471502</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>0.199</v>
+        <v>0.222</v>
       </c>
       <c r="G9" s="17">
         <f>MIN(1,F9*6)</f>
@@ -2334,17 +2341,17 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>0.6039720250584867</v>
+        <v>0.6040886323443799</v>
       </c>
       <c r="C10" s="18">
         <f>B10-$B$4</f>
         <v/>
       </c>
       <c r="D10" s="18" t="n">
-        <v>-0.193073361694687</v>
+        <v>-0.1931638302215448</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>-0.1254326788013387</v>
+        <v>-0.1255562405259627</v>
       </c>
       <c r="F10" s="17" t="n">
         <v>0.0005</v>
@@ -2361,17 +2368,17 @@
         </is>
       </c>
       <c r="B11" s="17" t="n">
-        <v>0.5311374036699636</v>
+        <v>0.5308164632739815</v>
       </c>
       <c r="C11" s="18">
         <f>B11-$B$4</f>
         <v/>
       </c>
       <c r="D11" s="18" t="n">
-        <v>-0.2815920991542617</v>
+        <v>-0.2817473419136437</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>-0.1812856158374114</v>
+        <v>-0.1825844403048875</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0.0005</v>
@@ -2462,7 +2469,7 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>0.6266128172318192</v>
+        <v>0.6263262473017398</v>
       </c>
       <c r="C4" s="18" t="n"/>
       <c r="D4" s="18" t="n"/>
@@ -2477,17 +2484,17 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>0.7525839350455473</v>
+        <v>0.7486232199110623</v>
       </c>
       <c r="C5" s="18">
         <f>B5-$B$4</f>
         <v/>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.0599783549713972</v>
+        <v>0.0585261873323647</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>0.1922636251348856</v>
+        <v>0.1877047383564628</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>0.0005</v>
@@ -2504,20 +2511,20 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>0.6812877022210035</v>
+        <v>0.6813926836151728</v>
       </c>
       <c r="C6" s="18">
         <f>B6-$B$4</f>
         <v/>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.008098410066950199</v>
+        <v>0.0099313294363728</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>0.1051822876724277</v>
+        <v>0.1038916185717283</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="G6" s="17">
         <f>MIN(1,F6*6)</f>
@@ -2531,17 +2538,17 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>0.7247547451482192</v>
+        <v>0.723652395444803</v>
       </c>
       <c r="C7" s="18">
         <f>B7-$B$4</f>
         <v/>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0.0493803501518459</v>
+        <v>0.048899444402803</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>0.1478544043325228</v>
+        <v>0.1454745818961373</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>0.0005</v>
@@ -2558,17 +2565,17 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>0.7307166468634799</v>
+        <v>0.7308909788486915</v>
       </c>
       <c r="C8" s="18">
         <f>B8-$B$4</f>
         <v/>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0.0596128290521198</v>
+        <v>0.0614331309447581</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>0.1479577248297307</v>
+        <v>0.1491328003599791</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>0.0005</v>
@@ -2585,20 +2592,20 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>0.667237912439448</v>
+        <v>0.6683218538096001</v>
       </c>
       <c r="C9" s="18">
         <f>B9-$B$4</f>
         <v/>
       </c>
       <c r="D9" s="18" t="n">
-        <v>-0.0119712517042226</v>
+        <v>-0.009500345591101101</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>0.09120181363480689</v>
+        <v>0.0913970209993212</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>0.115</v>
+        <v>0.114</v>
       </c>
       <c r="G9" s="17">
         <f>MIN(1,F9*6)</f>
@@ -2612,17 +2619,17 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>0.5680791670474972</v>
+        <v>0.5681544281976766</v>
       </c>
       <c r="C10" s="18">
         <f>B10-$B$4</f>
         <v/>
       </c>
       <c r="D10" s="18" t="n">
-        <v>-0.0905528171102274</v>
+        <v>-0.0898448854973109</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>-0.0278237792693648</v>
+        <v>-0.0278566423990828</v>
       </c>
       <c r="F10" s="17" t="n">
         <v>0.0005</v>
@@ -2639,17 +2646,17 @@
         </is>
       </c>
       <c r="B11" s="17" t="n">
-        <v>0.5052554611095877</v>
+        <v>0.5049808166098411</v>
       </c>
       <c r="C11" s="18">
         <f>B11-$B$4</f>
         <v/>
       </c>
       <c r="D11" s="18" t="n">
-        <v>-0.1712187264084851</v>
+        <v>-0.1706464804453073</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>-0.0753579660663876</v>
+        <v>-0.0752561959904862</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0.0005</v>
@@ -2735,13 +2742,13 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>0.7438354214123006</v>
+        <v>0.744479405034325</v>
       </c>
       <c r="C4" s="18" t="n"/>
       <c r="D4" s="18" t="n"/>
       <c r="E4" s="18" t="n"/>
       <c r="F4" s="17" t="n">
-        <v>0.6808182527590948</v>
+        <v>0.6812824051624454</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
@@ -2751,20 +2758,20 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>0.9111332574031891</v>
+        <v>0.9129290617848971</v>
       </c>
       <c r="C5" s="18">
         <f>B5-$B$4</f>
         <v/>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.07675753614260297</v>
+        <v>0.08221295117877488</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>0.2647359585531192</v>
+        <v>0.269027063788093</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.7084277804615213</v>
+        <v>0.708139057779104</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
@@ -2774,20 +2781,20 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>0.9035449886104784</v>
+        <v>0.9046481693363845</v>
       </c>
       <c r="C6" s="18">
         <f>B6-$B$4</f>
         <v/>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.06683609790819094</v>
+        <v>0.07139672690305819</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>0.25787137641433</v>
+        <v>0.2624006045581693</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.7272490803017353</v>
+        <v>0.7277966354582416</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
@@ -2797,20 +2804,20 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>0.8995017084282461</v>
+        <v>0.900729405034325</v>
       </c>
       <c r="C7" s="18">
         <f>B7-$B$4</f>
         <v/>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0.06314394120270203</v>
+        <v>0.06739960105840408</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>0.2586427139447331</v>
+        <v>0.2600384641319204</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0.6897736984876073</v>
+        <v>0.6902532731545377</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
@@ -2820,20 +2827,20 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>0.8905466970387244</v>
+        <v>0.8920051487414188</v>
       </c>
       <c r="C8" s="18">
         <f>B8-$B$4</f>
         <v/>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0.0446372700183863</v>
+        <v>0.05092867025429097</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>0.252442977628922</v>
+        <v>0.2555133972754777</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>0.7220931960908179</v>
+        <v>0.722471931067925</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
@@ -2843,7 +2850,7 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>0.7870159453302962</v>
+        <v>0.7885869565217392</v>
       </c>
       <c r="C9" s="18">
         <f>B9-$B$4</f>
@@ -2852,7 +2859,7 @@
       <c r="D9" s="18" t="n"/>
       <c r="E9" s="18" t="n"/>
       <c r="F9" s="17" t="n">
-        <v>0.6862621232953068</v>
+        <v>0.6876049087992838</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
@@ -2954,22 +2961,22 @@
         <v>66</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>0.6456748411210327</v>
+        <v>0.6436911049942966</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.9691742315951016</v>
+        <v>0.9695170299558598</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.9729874815131095</v>
+        <v>0.9734863983534195</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.9385009993750039</v>
+        <v>0.9388071591529037</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>0.9117301254323922</v>
+        <v>0.9120697564846501</v>
       </c>
       <c r="H5" t="n">
-        <v>0.978129776424651</v>
+        <v>0.9783994817239497</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
@@ -2982,22 +2989,22 @@
         <v>70</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>0.8580133609498526</v>
+        <v>0.8577890460603227</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.83640085766796</v>
+        <v>0.8361117605798457</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.8251101257329561</v>
+        <v>0.8255830605564649</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.8061825024067213</v>
+        <v>0.8065492751928923</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>0.8332244231161937</v>
+        <v>0.8335574000467616</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6893593745441817</v>
+        <v>0.6895063712882862</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
@@ -3010,22 +3017,22 @@
         <v>20</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>0.8875056156830713</v>
+        <v>0.8873782733224223</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>0.8865489074943843</v>
+        <v>0.8882815057283142</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.8698029405758628</v>
+        <v>0.8703508592471358</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0.922327955891362</v>
+        <v>0.9228662029459903</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>0.917623034510925</v>
+        <v>0.9179930441898527</v>
       </c>
       <c r="H7" t="n">
-        <v>0.779630385950582</v>
+        <v>0.7798895253682488</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
@@ -3038,22 +3045,22 @@
         <v>149</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>0.7632077165447135</v>
+        <v>0.7622047968453081</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>0.8972632196400208</v>
+        <v>0.897368366853766</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.8936871362140634</v>
+        <v>0.8941765342325816</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>0.8738226252753021</v>
+        <v>0.8741787860147848</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>0.8738756641855787</v>
+        <v>0.8742146223047266</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8242246656972562</v>
+        <v>0.8244365052340206</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
@@ -3079,22 +3086,22 @@
         <v>52</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>0.3772252879078695</v>
+        <v>0.377115754260156</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>0.7194460080466559</v>
+        <v>0.7201107548146231</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>0.5221329174664107</v>
+        <v>0.5221186190071342</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>0.649544607264137</v>
+        <v>0.6499362362769378</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.5951111029086078</v>
+        <v>0.595169666950061</v>
       </c>
       <c r="H10" t="n">
-        <v>0.61837673482947</v>
+        <v>0.6186259379736072</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
@@ -3107,22 +3114,22 @@
         <v>63</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>0.8066241659811716</v>
+        <v>0.8063644615302472</v>
       </c>
       <c r="D11" s="17" t="n">
-        <v>0.771337362520184</v>
+        <v>0.7695239620756199</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>0.8017339213356488</v>
+        <v>0.8019362638536112</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>0.7647804131249429</v>
+        <v>0.7654020121583793</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.829193705633245</v>
+        <v>0.8294585173489546</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6779297291533376</v>
+        <v>0.6782472559743102</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="11">
@@ -3135,22 +3142,22 @@
         <v>17</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>0.8065103872643107</v>
+        <v>0.8060166209684259</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>0.8503951676639947</v>
+        <v>0.8458659581083754</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>0.7664841368409168</v>
+        <v>0.7666280351640895</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>0.8593471265665575</v>
+        <v>0.8596460977471239</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.8259850965338151</v>
+        <v>0.8262147723096926</v>
       </c>
       <c r="H12" t="n">
-        <v>0.724398780625494</v>
+        <v>0.7247081437091897</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="11">
@@ -3163,22 +3170,22 @@
         <v>126</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>0.6267571519970752</v>
+        <v>0.6265344805229475</v>
       </c>
       <c r="D13" s="17" t="n">
-        <v>0.7554207415531792</v>
+        <v>0.7543851971350769</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>0.6812877022210035</v>
+        <v>0.6813926836151729</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>0.7264663878987296</v>
+        <v>0.7270260787319894</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.73071664686348</v>
+        <v>0.7308909788486915</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6538250616945434</v>
+        <v>0.6541116526700381</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="11">
@@ -3511,40 +3518,40 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.2295344679757571</v>
+        <v>0.2260938556329331</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02506581222288731</v>
+        <v>0.02509587285767527</v>
       </c>
       <c r="E4" t="n">
-        <v>1.086640234786473</v>
+        <v>1.061950333880051</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.02831372516967114</v>
+        <v>-0.04452900769718918</v>
       </c>
       <c r="G4" t="n">
-        <v>0.785234899328859</v>
+        <v>0.7986577181208053</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8462323871758219</v>
+        <v>0.8349018003273322</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1344827586206896</v>
+        <v>0.1285097192224622</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9923371647509579</v>
+        <v>0.9927025054731209</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.1838395870557872</v>
       </c>
       <c r="L4" t="n">
-        <v>0.006024573919936584</v>
+        <v>0.006075044669446099</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01080063416567578</v>
+        <v>0.01081993249950367</v>
       </c>
       <c r="N4" t="n">
-        <v>0.01603250099088387</v>
+        <v>0.01584276354973198</v>
       </c>
     </row>
     <row r="5">
@@ -3559,40 +3566,40 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.1844374990629637</v>
+        <v>0.1909887477220659</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02561585837572898</v>
+        <v>0.02561521339571764</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9879690002439582</v>
+        <v>0.9910934453263044</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.004322604940026632</v>
+        <v>-0.004639606923424779</v>
       </c>
       <c r="G5" t="n">
         <v>0.785234899328859</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8311210945476822</v>
+        <v>0.8316284779050737</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1239406779661017</v>
+        <v>0.124468085106383</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9921989273525109</v>
+        <v>0.9921894068830852</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1870788743559255</v>
+        <v>0.1866190192574946</v>
       </c>
       <c r="L5" t="n">
-        <v>0.002695204122076893</v>
+        <v>0.002898550724637682</v>
       </c>
       <c r="M5" t="n">
-        <v>0.009274673008323424</v>
+        <v>0.009688306531665674</v>
       </c>
       <c r="N5" t="n">
-        <v>0.01489298454221165</v>
+        <v>0.01493944808417709</v>
       </c>
     </row>
     <row r="6">
@@ -3607,40 +3614,40 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.1753661270949595</v>
+        <v>0.1757756231650459</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02597582725174593</v>
+        <v>0.02601064285968114</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9931475518719396</v>
+        <v>1.000281375080055</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.004774228210969339</v>
+        <v>-0.005540196552974494</v>
       </c>
       <c r="G6" t="n">
         <v>0.7919463087248322</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8427608740044925</v>
+        <v>0.8432896890343698</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1328828828828829</v>
+        <v>0.1334841628959276</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9925444925444925</v>
+        <v>0.9925355164941007</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1759809750297265</v>
+        <v>0.1755012904506651</v>
       </c>
       <c r="L6" t="n">
-        <v>0.002695204122076893</v>
+        <v>0.002938256898947787</v>
       </c>
       <c r="M6" t="n">
-        <v>0.008997225525168448</v>
+        <v>0.009410363311494935</v>
       </c>
       <c r="N6" t="n">
-        <v>0.01546769718588981</v>
+        <v>0.01549533452451856</v>
       </c>
     </row>
     <row r="7">
@@ -3655,40 +3662,40 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.1719750799692672</v>
+        <v>0.177752345432581</v>
       </c>
       <c r="D7" t="n">
-        <v>0.02603112214350956</v>
+        <v>0.0260426240749838</v>
       </c>
       <c r="E7" t="n">
-        <v>1.07206022415256</v>
+        <v>1.044173588866299</v>
       </c>
       <c r="F7" t="n">
-        <v>0.007250948427309378</v>
+        <v>-0.002184308929572658</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7919463087248322</v>
+        <v>0.8053691275167785</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8100878088625689</v>
+        <v>0.8038052373158756</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1125954198473282</v>
+        <v>0.1112140871177016</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9922461230615308</v>
+        <v>0.9926730672056594</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2076892588188664</v>
+        <v>0.2142148104030177</v>
       </c>
       <c r="L7" t="n">
-        <v>0.002338485929449069</v>
+        <v>0.002541195155846735</v>
       </c>
       <c r="M7" t="n">
-        <v>0.008085612366230677</v>
+        <v>0.008040500297796306</v>
       </c>
       <c r="N7" t="n">
-        <v>0.01439754260800634</v>
+        <v>0.01453245979749851</v>
       </c>
     </row>
     <row r="8">
@@ -3703,40 +3710,40 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.1112965384710407</v>
+        <v>0.1111358820093567</v>
       </c>
       <c r="D8" t="n">
-        <v>0.02752650275823896</v>
+        <v>0.02758077382032902</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9913595502153402</v>
+        <v>0.9910986255443853</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.005980251387520434</v>
+        <v>-0.00614317333440432</v>
       </c>
       <c r="G8" t="n">
         <v>0.7986577181208053</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5699407800694303</v>
+        <v>0.5683306055646481</v>
       </c>
       <c r="I8" t="n">
-        <v>0.05348314606741573</v>
+        <v>0.05338716913414087</v>
       </c>
       <c r="J8" t="n">
-        <v>0.989365473236441</v>
+        <v>0.9893162393162394</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4409433214427269</v>
+        <v>0.4425253126861227</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.003032104637336504</v>
+        <v>0.00311693468334326</v>
       </c>
       <c r="N8" t="n">
-        <v>0.008531510107015458</v>
+        <v>0.008606313281715306</v>
       </c>
     </row>
     <row r="9">
@@ -3751,40 +3758,40 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.09476579481990252</v>
+        <v>0.0964939401633446</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02777774711172786</v>
+        <v>0.02779353938686501</v>
       </c>
       <c r="E9" t="n">
-        <v>1.075469920058045</v>
+        <v>1.097043873635803</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01462486734399807</v>
+        <v>0.02030759801655716</v>
       </c>
       <c r="G9" t="n">
         <v>0.8187919463087249</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4617112517868083</v>
+        <v>0.478518821603928</v>
       </c>
       <c r="I9" t="n">
-        <v>0.04423495286439449</v>
+        <v>0.04567577686259828</v>
       </c>
       <c r="J9" t="n">
-        <v>0.9881993006993007</v>
+        <v>0.9885883347421809</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5465715418152992</v>
+        <v>0.5302759579114552</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>0.001149425287356322</v>
+        <v>0.001111772880682946</v>
       </c>
       <c r="N9" t="n">
-        <v>0.009373761395164486</v>
+        <v>0.009797498511018464</v>
       </c>
     </row>
     <row r="10">
@@ -3799,10 +3806,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.02952833927863655</v>
+        <v>0.02958109986102839</v>
       </c>
       <c r="D10" t="n">
-        <v>0.02865641645808228</v>
+        <v>0.02870605839204026</v>
       </c>
     </row>
     <row r="11">
@@ -3817,40 +3824,40 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.08521677951450135</v>
+        <v>0.0834551039518848</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02766025850960952</v>
+        <v>0.02771763624468854</v>
       </c>
       <c r="E11" t="n">
-        <v>1.158922573673336</v>
+        <v>1.126749284542437</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.06657935493350987</v>
+        <v>-0.06861016047518335</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8412698412698413</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4992802303262956</v>
+        <v>0.4812590100913023</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0479014598540146</v>
+        <v>0.0467991169977925</v>
       </c>
       <c r="J11" t="n">
-        <v>0.9900095147478591</v>
+        <v>0.9901136925358379</v>
       </c>
       <c r="K11" t="n">
-        <v>0.5104797391709361</v>
+        <v>0.5282182835820896</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0003493246390312063</v>
+        <v>0.0001632462686567163</v>
       </c>
       <c r="N11" t="n">
-        <v>0.00716115510013973</v>
+        <v>0.006879664179104478</v>
       </c>
     </row>
     <row r="12">
@@ -3865,31 +3872,31 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.05062672744829048</v>
+        <v>0.05080242202151385</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02815802062181195</v>
+        <v>0.02819394089268755</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9483481095724542</v>
+        <v>0.9492716860715495</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.004682623198508686</v>
+        <v>-0.004547980005142629</v>
       </c>
       <c r="G12" t="n">
         <v>0.8015873015873016</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4517754318618042</v>
+        <v>0.4514656415185007</v>
       </c>
       <c r="I12" t="n">
-        <v>0.04233025984911987</v>
+        <v>0.04236577181208054</v>
       </c>
       <c r="J12" t="n">
-        <v>0.9868972746331237</v>
+        <v>0.9868697478991597</v>
       </c>
       <c r="K12" t="n">
-        <v>0.5556590591523055</v>
+        <v>0.5559701492537313</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -3898,7 +3905,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.003446669771774569</v>
+        <v>0.003404850746268657</v>
       </c>
     </row>
     <row r="13">
@@ -3913,40 +3920,40 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.0657719994412717</v>
+        <v>0.06629201704736558</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02788264124527806</v>
+        <v>0.02791688164067146</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9751588747917186</v>
+        <v>0.975656516732223</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.002241119276739794</v>
+        <v>-0.00212486915810384</v>
       </c>
       <c r="G13" t="n">
         <v>0.8015873015873016</v>
       </c>
       <c r="H13" t="n">
-        <v>0.5890115163147792</v>
+        <v>0.5888995675156175</v>
       </c>
       <c r="I13" t="n">
-        <v>0.05567805953693495</v>
+        <v>0.05573951434878587</v>
       </c>
       <c r="J13" t="n">
-        <v>0.9899193548387096</v>
+        <v>0.9899030694668821</v>
       </c>
       <c r="K13" t="n">
-        <v>0.4224499301350722</v>
+        <v>0.4225746268656717</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.0006054960409874245</v>
+        <v>-0.0006529850746268656</v>
       </c>
       <c r="N13" t="n">
-        <v>0.004413134606427572</v>
+        <v>0.004407649253731343</v>
       </c>
     </row>
     <row r="14">
@@ -3961,40 +3968,40 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0644946967358081</v>
+        <v>0.0645729000927288</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02788026651722164</v>
+        <v>0.02792098909106</v>
       </c>
       <c r="E14" t="n">
-        <v>1.075412988199589</v>
+        <v>1.026583957358763</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.008215222846687494</v>
+        <v>-0.01449830602781368</v>
       </c>
       <c r="G14" t="n">
         <v>0.7936507936507936</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5328694817658349</v>
+        <v>0.5321960595867371</v>
       </c>
       <c r="I14" t="n">
         <v>0.04885197850512946</v>
       </c>
       <c r="J14" t="n">
-        <v>0.9884290164663997</v>
+        <v>0.9883980365908077</v>
       </c>
       <c r="K14" t="n">
-        <v>0.4767116907312529</v>
+        <v>0.4773787313432836</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.000232883092687471</v>
+        <v>-0.0006296641791044776</v>
       </c>
       <c r="N14" t="n">
-        <v>0.006590591523055425</v>
+        <v>0.006553171641791043</v>
       </c>
     </row>
     <row r="15">
@@ -4009,31 +4016,31 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.05391257689226329</v>
+        <v>0.05389450429240197</v>
       </c>
       <c r="D15" t="n">
-        <v>0.02829360358512675</v>
+        <v>0.0283328505785215</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9153978808503124</v>
+        <v>0.9144827459128204</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.001851267795798534</v>
+        <v>-0.001971924974016033</v>
       </c>
       <c r="G15" t="n">
         <v>0.7936507936507936</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2881477927063339</v>
+        <v>0.2854396924555502</v>
       </c>
       <c r="I15" t="n">
-        <v>0.032605151613955</v>
+        <v>0.03253090435914118</v>
       </c>
       <c r="J15" t="n">
-        <v>0.9788101059494703</v>
+        <v>0.9785831960461285</v>
       </c>
       <c r="K15" t="n">
-        <v>0.7142524452724732</v>
+        <v>0.7168843283582089</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -4042,7 +4049,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0.003435025617140196</v>
+        <v>0.003696361940298507</v>
       </c>
     </row>
     <row r="16">
@@ -4057,31 +4064,31 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.06037014219553517</v>
+        <v>0.07288011479741094</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02812598530144687</v>
+        <v>0.02813427461858303</v>
       </c>
       <c r="E16" t="n">
-        <v>1.260703044771871</v>
+        <v>1.109318674513565</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.008544417368427756</v>
+        <v>-0.0114528663555734</v>
       </c>
       <c r="G16" t="n">
-        <v>0.8492063492063492</v>
+        <v>0.8253968253968254</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2922264875239923</v>
+        <v>0.3087457952907256</v>
       </c>
       <c r="I16" t="n">
-        <v>0.03500163559044815</v>
+        <v>0.03488762160348876</v>
       </c>
       <c r="J16" t="n">
-        <v>0.98464025869038</v>
+        <v>0.9831675592960979</v>
       </c>
       <c r="K16" t="n">
-        <v>0.7119236143455985</v>
+        <v>0.695195895522388</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -4090,7 +4097,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0.004843968327899395</v>
+        <v>0.004967350746268656</v>
       </c>
     </row>
     <row r="17">
@@ -4105,10 +4112,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.02934326967862133</v>
+        <v>0.02938432835820896</v>
       </c>
       <c r="D17" t="n">
-        <v>0.02848224220318903</v>
+        <v>0.02852088960514591</v>
       </c>
     </row>
     <row r="19">
@@ -4187,22 +4194,22 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>5046</v>
+        <v>5037</v>
       </c>
       <c r="C4" s="20" t="n">
         <v>149</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>0.7632077165447135</v>
+        <v>0.7622047968453081</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>0.8972632196400208</v>
+        <v>0.897368366853766</v>
       </c>
       <c r="F4" s="17" t="n">
-        <v>0.8936871362140634</v>
+        <v>0.8941765342325816</v>
       </c>
       <c r="G4" s="17" t="n">
-        <v>0.8738226252753021</v>
+        <v>0.8741787860147848</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
@@ -4212,22 +4219,22 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>4980</v>
+        <v>4971</v>
       </c>
       <c r="C5" s="20" t="n">
         <v>83</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.8566675933876409</v>
+        <v>0.8564446000039438</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.8571074988128951</v>
+        <v>0.856293627866622</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.8306290303136171</v>
+        <v>0.8311108591485418</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>0.856184632341906</v>
+        <v>0.8573874055961982</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
@@ -4237,22 +4244,22 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>5575</v>
+        <v>5566</v>
       </c>
       <c r="C6" s="20" t="n">
         <v>81</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.8890547263681592</v>
+        <v>0.8888249659565369</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.9541473976099629</v>
+        <v>0.9544558110222041</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.9000357292130137</v>
+        <v>0.900481672800117</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>0.9318841654419862</v>
+        <v>0.9327708565447855</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
@@ -4338,22 +4345,22 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>5046</v>
+        <v>5037</v>
       </c>
       <c r="C4" s="20" t="n">
         <v>149</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>0.7642673983386623</v>
+        <v>0.76321274398884</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>0.8752530312353954</v>
+        <v>0.8767190434868573</v>
       </c>
       <c r="F4" s="17" t="n">
-        <v>0.8936871362140634</v>
+        <v>0.8941765342325816</v>
       </c>
       <c r="G4" s="17" t="n">
-        <v>0.8738756641855786</v>
+        <v>0.8742146223047266</v>
       </c>
       <c r="H4" s="18">
         <f>E4-D4</f>
@@ -4367,22 +4374,22 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>5035</v>
+        <v>5026</v>
       </c>
       <c r="C5" s="20" t="n">
         <v>138</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0.7592063167925941</v>
+        <v>0.758067672383121</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.875920779655098</v>
+        <v>0.8766173889323751</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.8980194913774479</v>
+        <v>0.8985062501482483</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>0.873017493703628</v>
+        <v>0.8733499964420408</v>
       </c>
       <c r="H5" s="18">
         <f>E5-D5</f>
@@ -4396,22 +4403,22 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>4629</v>
+        <v>4620</v>
       </c>
       <c r="C6" s="20" t="n">
         <v>130</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.7893241233094533</v>
+        <v>0.7882730854891211</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.8970848222681963</v>
+        <v>0.8945057392496145</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.9065142681279601</v>
+        <v>0.9070806921363714</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>0.8868004855779917</v>
+        <v>0.887205756381703</v>
       </c>
       <c r="H6" s="18">
         <f>E6-D6</f>
@@ -4425,22 +4432,22 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>5055</v>
+        <v>5046</v>
       </c>
       <c r="C7" s="20" t="n">
         <v>158</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>0.7705428019738254</v>
+        <v>0.7695272845925957</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.8796395623256812</v>
+        <v>0.879915162941018</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0.8962235985348819</v>
+        <v>0.8967161894797904</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>0.876524764580743</v>
+        <v>0.8768554869585033</v>
       </c>
       <c r="H7" s="18">
         <f>E7-D7</f>
@@ -4454,22 +4461,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5057</v>
+        <v>5048</v>
       </c>
       <c r="C8" t="n">
         <v>160</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7618031447825199</v>
+        <v>0.7607853416530278</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8717365223606289</v>
+        <v>0.8720335515548282</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8885829334286298</v>
+        <v>0.8890669752454992</v>
       </c>
       <c r="G8" t="n">
-        <v>0.8708890647335104</v>
+        <v>0.871219056873977</v>
       </c>
       <c r="H8">
         <f>E8-D8</f>
@@ -4483,22 +4490,22 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>4201</v>
+        <v>4193</v>
       </c>
       <c r="C9" s="20" t="n">
         <v>104</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>0.744979910253281</v>
+        <v>0.743632071034859</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>0.8900461876419894</v>
+        <v>0.8905764998024719</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>0.9097662924090798</v>
+        <v>0.9102787497413323</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>0.8922499577552055</v>
+        <v>0.8926811144345994</v>
       </c>
       <c r="H9" s="18">
         <f>E9-D9</f>

</xml_diff>